<commit_message>
Speed up workbook formulas with helper columns
LibreOffice could not finish recalculating the first build inside 9 minutes,
which meant no formula in it could be verified before shipping.

Two hot spots, both from recomputing the same subexpression repeatedly:

- Client Matcher evaluated COUNTIF across the client list three times per row
  (once to test for zero, once for the ambiguity test, once to interpolate the
  number). It now counts once into its own column and reads that back.
- Money in Words re-derived each INT/MOD digit-group expression inside every
  INDEX call, so a single cell held four copies of a nested arithmetic
  expression. The groups and their words now live in their own columns, which
  also makes a wrong answer traceable to one step.

Heavy-formula row counts trimmed to 40/30/20, which is well past what these
sheets are used for at once.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CyctpJscZQ6yHKvMF9mzPQ
</commit_message>
<xml_diff>
--- a/AkhiSal-Tools.xlsx
+++ b/AkhiSal-Tools.xlsx
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,6 +156,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2075,7 +2076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2083,6 +2084,7 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2125,6 +2127,11 @@
           <t>Result</t>
         </is>
       </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -2145,7 +2152,11 @@
         <v/>
       </c>
       <c r="E4" s="10">
-        <f>IF($B4="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B4)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B4)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B4)&amp;" clients share this name","matched")))</f>
+        <f>IF($B4="","",IF($F4=0,"no match - new client, or a typo",IF($F4&gt;1,"CHECK PHONE - "&amp;$F4&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F4" s="11">
+        <f>IF($B4="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B4))</f>
         <v/>
       </c>
     </row>
@@ -2168,7 +2179,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>IF($B5="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B5)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B5)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B5)&amp;" clients share this name","matched")))</f>
+        <f>IF($B5="","",IF($F5=0,"no match - new client, or a typo",IF($F5&gt;1,"CHECK PHONE - "&amp;$F5&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F5" s="11">
+        <f>IF($B5="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B5))</f>
         <v/>
       </c>
     </row>
@@ -2191,7 +2206,11 @@
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>IF($B6="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B6)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B6)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B6)&amp;" clients share this name","matched")))</f>
+        <f>IF($B6="","",IF($F6=0,"no match - new client, or a typo",IF($F6&gt;1,"CHECK PHONE - "&amp;$F6&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>IF($B6="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B6))</f>
         <v/>
       </c>
     </row>
@@ -2214,7 +2233,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>IF($B7="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B7)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B7)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B7)&amp;" clients share this name","matched")))</f>
+        <f>IF($B7="","",IF($F7=0,"no match - new client, or a typo",IF($F7&gt;1,"CHECK PHONE - "&amp;$F7&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F7" s="11">
+        <f>IF($B7="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B7))</f>
         <v/>
       </c>
     </row>
@@ -2237,7 +2260,11 @@
         <v/>
       </c>
       <c r="E8" s="10">
-        <f>IF($B8="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B8)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B8)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B8)&amp;" clients share this name","matched")))</f>
+        <f>IF($B8="","",IF($F8=0,"no match - new client, or a typo",IF($F8&gt;1,"CHECK PHONE - "&amp;$F8&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F8" s="11">
+        <f>IF($B8="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B8))</f>
         <v/>
       </c>
     </row>
@@ -2260,7 +2287,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>IF($B9="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B9)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B9)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B9)&amp;" clients share this name","matched")))</f>
+        <f>IF($B9="","",IF($F9=0,"no match - new client, or a typo",IF($F9&gt;1,"CHECK PHONE - "&amp;$F9&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F9" s="11">
+        <f>IF($B9="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B9))</f>
         <v/>
       </c>
     </row>
@@ -2279,7 +2310,11 @@
         <v/>
       </c>
       <c r="E10" s="10">
-        <f>IF($B10="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B10)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B10)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B10)&amp;" clients share this name","matched")))</f>
+        <f>IF($B10="","",IF($F10=0,"no match - new client, or a typo",IF($F10&gt;1,"CHECK PHONE - "&amp;$F10&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F10" s="11">
+        <f>IF($B10="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B10))</f>
         <v/>
       </c>
     </row>
@@ -2298,7 +2333,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>IF($B11="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B11)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B11)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B11)&amp;" clients share this name","matched")))</f>
+        <f>IF($B11="","",IF($F11=0,"no match - new client, or a typo",IF($F11&gt;1,"CHECK PHONE - "&amp;$F11&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F11" s="11">
+        <f>IF($B11="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B11))</f>
         <v/>
       </c>
     </row>
@@ -2317,7 +2356,11 @@
         <v/>
       </c>
       <c r="E12" s="10">
-        <f>IF($B12="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B12)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B12)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B12)&amp;" clients share this name","matched")))</f>
+        <f>IF($B12="","",IF($F12=0,"no match - new client, or a typo",IF($F12&gt;1,"CHECK PHONE - "&amp;$F12&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F12" s="11">
+        <f>IF($B12="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B12))</f>
         <v/>
       </c>
     </row>
@@ -2336,7 +2379,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>IF($B13="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B13)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B13)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B13)&amp;" clients share this name","matched")))</f>
+        <f>IF($B13="","",IF($F13=0,"no match - new client, or a typo",IF($F13&gt;1,"CHECK PHONE - "&amp;$F13&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F13" s="11">
+        <f>IF($B13="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B13))</f>
         <v/>
       </c>
     </row>
@@ -2355,7 +2402,11 @@
         <v/>
       </c>
       <c r="E14" s="10">
-        <f>IF($B14="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B14)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B14)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B14)&amp;" clients share this name","matched")))</f>
+        <f>IF($B14="","",IF($F14=0,"no match - new client, or a typo",IF($F14&gt;1,"CHECK PHONE - "&amp;$F14&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F14" s="11">
+        <f>IF($B14="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B14))</f>
         <v/>
       </c>
     </row>
@@ -2374,7 +2425,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>IF($B15="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B15)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B15)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B15)&amp;" clients share this name","matched")))</f>
+        <f>IF($B15="","",IF($F15=0,"no match - new client, or a typo",IF($F15&gt;1,"CHECK PHONE - "&amp;$F15&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F15" s="11">
+        <f>IF($B15="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B15))</f>
         <v/>
       </c>
     </row>
@@ -2393,7 +2448,11 @@
         <v/>
       </c>
       <c r="E16" s="10">
-        <f>IF($B16="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B16)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B16)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B16)&amp;" clients share this name","matched")))</f>
+        <f>IF($B16="","",IF($F16=0,"no match - new client, or a typo",IF($F16&gt;1,"CHECK PHONE - "&amp;$F16&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F16" s="11">
+        <f>IF($B16="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B16))</f>
         <v/>
       </c>
     </row>
@@ -2412,7 +2471,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IF($B17="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B17)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B17)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B17)&amp;" clients share this name","matched")))</f>
+        <f>IF($B17="","",IF($F17=0,"no match - new client, or a typo",IF($F17&gt;1,"CHECK PHONE - "&amp;$F17&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F17" s="11">
+        <f>IF($B17="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B17))</f>
         <v/>
       </c>
     </row>
@@ -2431,7 +2494,11 @@
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IF($B18="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B18)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B18)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B18)&amp;" clients share this name","matched")))</f>
+        <f>IF($B18="","",IF($F18=0,"no match - new client, or a typo",IF($F18&gt;1,"CHECK PHONE - "&amp;$F18&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F18" s="11">
+        <f>IF($B18="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B18))</f>
         <v/>
       </c>
     </row>
@@ -2450,7 +2517,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IF($B19="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B19)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B19)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B19)&amp;" clients share this name","matched")))</f>
+        <f>IF($B19="","",IF($F19=0,"no match - new client, or a typo",IF($F19&gt;1,"CHECK PHONE - "&amp;$F19&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F19" s="11">
+        <f>IF($B19="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B19))</f>
         <v/>
       </c>
     </row>
@@ -2469,7 +2540,11 @@
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>IF($B20="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B20)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B20)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B20)&amp;" clients share this name","matched")))</f>
+        <f>IF($B20="","",IF($F20=0,"no match - new client, or a typo",IF($F20&gt;1,"CHECK PHONE - "&amp;$F20&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F20" s="11">
+        <f>IF($B20="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B20))</f>
         <v/>
       </c>
     </row>
@@ -2488,7 +2563,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>IF($B21="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B21)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B21)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B21)&amp;" clients share this name","matched")))</f>
+        <f>IF($B21="","",IF($F21=0,"no match - new client, or a typo",IF($F21&gt;1,"CHECK PHONE - "&amp;$F21&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F21" s="11">
+        <f>IF($B21="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B21))</f>
         <v/>
       </c>
     </row>
@@ -2507,7 +2586,11 @@
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>IF($B22="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B22)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B22)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B22)&amp;" clients share this name","matched")))</f>
+        <f>IF($B22="","",IF($F22=0,"no match - new client, or a typo",IF($F22&gt;1,"CHECK PHONE - "&amp;$F22&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F22" s="11">
+        <f>IF($B22="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B22))</f>
         <v/>
       </c>
     </row>
@@ -2526,7 +2609,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>IF($B23="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B23)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B23)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B23)&amp;" clients share this name","matched")))</f>
+        <f>IF($B23="","",IF($F23=0,"no match - new client, or a typo",IF($F23&gt;1,"CHECK PHONE - "&amp;$F23&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F23" s="11">
+        <f>IF($B23="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B23))</f>
         <v/>
       </c>
     </row>
@@ -2545,7 +2632,11 @@
         <v/>
       </c>
       <c r="E24" s="10">
-        <f>IF($B24="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B24)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B24)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B24)&amp;" clients share this name","matched")))</f>
+        <f>IF($B24="","",IF($F24=0,"no match - new client, or a typo",IF($F24&gt;1,"CHECK PHONE - "&amp;$F24&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F24" s="11">
+        <f>IF($B24="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B24))</f>
         <v/>
       </c>
     </row>
@@ -2564,7 +2655,11 @@
         <v/>
       </c>
       <c r="E25" s="10">
-        <f>IF($B25="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B25)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B25)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B25)&amp;" clients share this name","matched")))</f>
+        <f>IF($B25="","",IF($F25=0,"no match - new client, or a typo",IF($F25&gt;1,"CHECK PHONE - "&amp;$F25&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F25" s="11">
+        <f>IF($B25="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B25))</f>
         <v/>
       </c>
     </row>
@@ -2583,7 +2678,11 @@
         <v/>
       </c>
       <c r="E26" s="10">
-        <f>IF($B26="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B26)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B26)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B26)&amp;" clients share this name","matched")))</f>
+        <f>IF($B26="","",IF($F26=0,"no match - new client, or a typo",IF($F26&gt;1,"CHECK PHONE - "&amp;$F26&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F26" s="11">
+        <f>IF($B26="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B26))</f>
         <v/>
       </c>
     </row>
@@ -2602,7 +2701,11 @@
         <v/>
       </c>
       <c r="E27" s="10">
-        <f>IF($B27="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B27)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B27)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B27)&amp;" clients share this name","matched")))</f>
+        <f>IF($B27="","",IF($F27=0,"no match - new client, or a typo",IF($F27&gt;1,"CHECK PHONE - "&amp;$F27&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F27" s="11">
+        <f>IF($B27="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B27))</f>
         <v/>
       </c>
     </row>
@@ -2621,7 +2724,11 @@
         <v/>
       </c>
       <c r="E28" s="10">
-        <f>IF($B28="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B28)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B28)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B28)&amp;" clients share this name","matched")))</f>
+        <f>IF($B28="","",IF($F28=0,"no match - new client, or a typo",IF($F28&gt;1,"CHECK PHONE - "&amp;$F28&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F28" s="11">
+        <f>IF($B28="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B28))</f>
         <v/>
       </c>
     </row>
@@ -2640,7 +2747,11 @@
         <v/>
       </c>
       <c r="E29" s="10">
-        <f>IF($B29="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B29)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B29)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B29)&amp;" clients share this name","matched")))</f>
+        <f>IF($B29="","",IF($F29=0,"no match - new client, or a typo",IF($F29&gt;1,"CHECK PHONE - "&amp;$F29&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F29" s="11">
+        <f>IF($B29="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B29))</f>
         <v/>
       </c>
     </row>
@@ -2659,7 +2770,11 @@
         <v/>
       </c>
       <c r="E30" s="10">
-        <f>IF($B30="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B30)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B30)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B30)&amp;" clients share this name","matched")))</f>
+        <f>IF($B30="","",IF($F30=0,"no match - new client, or a typo",IF($F30&gt;1,"CHECK PHONE - "&amp;$F30&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F30" s="11">
+        <f>IF($B30="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B30))</f>
         <v/>
       </c>
     </row>
@@ -2678,7 +2793,11 @@
         <v/>
       </c>
       <c r="E31" s="10">
-        <f>IF($B31="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B31)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B31)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B31)&amp;" clients share this name","matched")))</f>
+        <f>IF($B31="","",IF($F31=0,"no match - new client, or a typo",IF($F31&gt;1,"CHECK PHONE - "&amp;$F31&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F31" s="11">
+        <f>IF($B31="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B31))</f>
         <v/>
       </c>
     </row>
@@ -2697,7 +2816,11 @@
         <v/>
       </c>
       <c r="E32" s="10">
-        <f>IF($B32="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B32)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B32)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B32)&amp;" clients share this name","matched")))</f>
+        <f>IF($B32="","",IF($F32=0,"no match - new client, or a typo",IF($F32&gt;1,"CHECK PHONE - "&amp;$F32&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F32" s="11">
+        <f>IF($B32="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B32))</f>
         <v/>
       </c>
     </row>
@@ -2716,7 +2839,11 @@
         <v/>
       </c>
       <c r="E33" s="10">
-        <f>IF($B33="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B33)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B33)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B33)&amp;" clients share this name","matched")))</f>
+        <f>IF($B33="","",IF($F33=0,"no match - new client, or a typo",IF($F33&gt;1,"CHECK PHONE - "&amp;$F33&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F33" s="11">
+        <f>IF($B33="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B33))</f>
         <v/>
       </c>
     </row>
@@ -2735,7 +2862,11 @@
         <v/>
       </c>
       <c r="E34" s="10">
-        <f>IF($B34="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B34)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B34)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B34)&amp;" clients share this name","matched")))</f>
+        <f>IF($B34="","",IF($F34=0,"no match - new client, or a typo",IF($F34&gt;1,"CHECK PHONE - "&amp;$F34&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F34" s="11">
+        <f>IF($B34="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B34))</f>
         <v/>
       </c>
     </row>
@@ -2754,7 +2885,11 @@
         <v/>
       </c>
       <c r="E35" s="10">
-        <f>IF($B35="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B35)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B35)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B35)&amp;" clients share this name","matched")))</f>
+        <f>IF($B35="","",IF($F35=0,"no match - new client, or a typo",IF($F35&gt;1,"CHECK PHONE - "&amp;$F35&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F35" s="11">
+        <f>IF($B35="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B35))</f>
         <v/>
       </c>
     </row>
@@ -2773,7 +2908,11 @@
         <v/>
       </c>
       <c r="E36" s="10">
-        <f>IF($B36="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B36)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B36)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B36)&amp;" clients share this name","matched")))</f>
+        <f>IF($B36="","",IF($F36=0,"no match - new client, or a typo",IF($F36&gt;1,"CHECK PHONE - "&amp;$F36&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F36" s="11">
+        <f>IF($B36="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B36))</f>
         <v/>
       </c>
     </row>
@@ -2792,7 +2931,11 @@
         <v/>
       </c>
       <c r="E37" s="10">
-        <f>IF($B37="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B37)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B37)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B37)&amp;" clients share this name","matched")))</f>
+        <f>IF($B37="","",IF($F37=0,"no match - new client, or a typo",IF($F37&gt;1,"CHECK PHONE - "&amp;$F37&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F37" s="11">
+        <f>IF($B37="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B37))</f>
         <v/>
       </c>
     </row>
@@ -2811,7 +2954,11 @@
         <v/>
       </c>
       <c r="E38" s="10">
-        <f>IF($B38="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B38)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B38)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B38)&amp;" clients share this name","matched")))</f>
+        <f>IF($B38="","",IF($F38=0,"no match - new client, or a typo",IF($F38&gt;1,"CHECK PHONE - "&amp;$F38&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F38" s="11">
+        <f>IF($B38="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B38))</f>
         <v/>
       </c>
     </row>
@@ -2830,7 +2977,11 @@
         <v/>
       </c>
       <c r="E39" s="10">
-        <f>IF($B39="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B39)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B39)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B39)&amp;" clients share this name","matched")))</f>
+        <f>IF($B39="","",IF($F39=0,"no match - new client, or a typo",IF($F39&gt;1,"CHECK PHONE - "&amp;$F39&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F39" s="11">
+        <f>IF($B39="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B39))</f>
         <v/>
       </c>
     </row>
@@ -2849,7 +3000,11 @@
         <v/>
       </c>
       <c r="E40" s="10">
-        <f>IF($B40="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B40)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B40)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B40)&amp;" clients share this name","matched")))</f>
+        <f>IF($B40="","",IF($F40=0,"no match - new client, or a typo",IF($F40&gt;1,"CHECK PHONE - "&amp;$F40&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F40" s="11">
+        <f>IF($B40="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B40))</f>
         <v/>
       </c>
     </row>
@@ -2868,7 +3023,11 @@
         <v/>
       </c>
       <c r="E41" s="10">
-        <f>IF($B41="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B41)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B41)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B41)&amp;" clients share this name","matched")))</f>
+        <f>IF($B41="","",IF($F41=0,"no match - new client, or a typo",IF($F41&gt;1,"CHECK PHONE - "&amp;$F41&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F41" s="11">
+        <f>IF($B41="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B41))</f>
         <v/>
       </c>
     </row>
@@ -2887,7 +3046,11 @@
         <v/>
       </c>
       <c r="E42" s="10">
-        <f>IF($B42="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B42)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B42)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B42)&amp;" clients share this name","matched")))</f>
+        <f>IF($B42="","",IF($F42=0,"no match - new client, or a typo",IF($F42&gt;1,"CHECK PHONE - "&amp;$F42&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F42" s="11">
+        <f>IF($B42="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B42))</f>
         <v/>
       </c>
     </row>
@@ -2906,392 +3069,16 @@
         <v/>
       </c>
       <c r="E43" s="10">
-        <f>IF($B43="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B43)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B43)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B43)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="12" t="n"/>
-      <c r="B44" s="10">
-        <f>IF($A44="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A44),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C44" s="10">
-        <f>IF($B44="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B44,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D44" s="13">
-        <f>IF($B44="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B44,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E44" s="10">
-        <f>IF($B44="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B44)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B44)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B44)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="12" t="n"/>
-      <c r="B45" s="10">
-        <f>IF($A45="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A45),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C45" s="10">
-        <f>IF($B45="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B45,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D45" s="13">
-        <f>IF($B45="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B45,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E45" s="10">
-        <f>IF($B45="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B45)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B45)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B45)&amp;" clients share this name","matched")))</f>
+        <f>IF($B43="","",IF($F43=0,"no match - new client, or a typo",IF($F43&gt;1,"CHECK PHONE - "&amp;$F43&amp;" clients share this name","matched")))</f>
+        <v/>
+      </c>
+      <c r="F43" s="11">
+        <f>IF($B43="","",COUNTIF('CRM Clients'!$D$4:$D$53,$B43))</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="n"/>
-      <c r="B46" s="10">
-        <f>IF($A46="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A46),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C46" s="10">
-        <f>IF($B46="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B46,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D46" s="13">
-        <f>IF($B46="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B46,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E46" s="10">
-        <f>IF($B46="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B46)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B46)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B46)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="12" t="n"/>
-      <c r="B47" s="10">
-        <f>IF($A47="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A47),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C47" s="10">
-        <f>IF($B47="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B47,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D47" s="13">
-        <f>IF($B47="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B47,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E47" s="10">
-        <f>IF($B47="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B47)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B47)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B47)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="12" t="n"/>
-      <c r="B48" s="10">
-        <f>IF($A48="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A48),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C48" s="10">
-        <f>IF($B48="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B48,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D48" s="13">
-        <f>IF($B48="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B48,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E48" s="10">
-        <f>IF($B48="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B48)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B48)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B48)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="12" t="n"/>
-      <c r="B49" s="10">
-        <f>IF($A49="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A49),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C49" s="10">
-        <f>IF($B49="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B49,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D49" s="13">
-        <f>IF($B49="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B49,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E49" s="10">
-        <f>IF($B49="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B49)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B49)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B49)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="12" t="n"/>
-      <c r="B50" s="10">
-        <f>IF($A50="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A50),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C50" s="10">
-        <f>IF($B50="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B50,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D50" s="13">
-        <f>IF($B50="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B50,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E50" s="10">
-        <f>IF($B50="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B50)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B50)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B50)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="12" t="n"/>
-      <c r="B51" s="10">
-        <f>IF($A51="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A51),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C51" s="10">
-        <f>IF($B51="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B51,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D51" s="13">
-        <f>IF($B51="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B51,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E51" s="10">
-        <f>IF($B51="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B51)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B51)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B51)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="12" t="n"/>
-      <c r="B52" s="10">
-        <f>IF($A52="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A52),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C52" s="10">
-        <f>IF($B52="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B52,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D52" s="13">
-        <f>IF($B52="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B52,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E52" s="10">
-        <f>IF($B52="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B52)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B52)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B52)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="12" t="n"/>
-      <c r="B53" s="10">
-        <f>IF($A53="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A53),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C53" s="10">
-        <f>IF($B53="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B53,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D53" s="13">
-        <f>IF($B53="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B53,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E53" s="10">
-        <f>IF($B53="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B53)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B53)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B53)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="12" t="n"/>
-      <c r="B54" s="10">
-        <f>IF($A54="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A54),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C54" s="10">
-        <f>IF($B54="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B54,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D54" s="13">
-        <f>IF($B54="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B54,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E54" s="10">
-        <f>IF($B54="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B54)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B54)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B54)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="12" t="n"/>
-      <c r="B55" s="10">
-        <f>IF($A55="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A55),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C55" s="10">
-        <f>IF($B55="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B55,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D55" s="13">
-        <f>IF($B55="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B55,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E55" s="10">
-        <f>IF($B55="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B55)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B55)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B55)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="12" t="n"/>
-      <c r="B56" s="10">
-        <f>IF($A56="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A56),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C56" s="10">
-        <f>IF($B56="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B56,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D56" s="13">
-        <f>IF($B56="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B56,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E56" s="10">
-        <f>IF($B56="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B56)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B56)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B56)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="12" t="n"/>
-      <c r="B57" s="10">
-        <f>IF($A57="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A57),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C57" s="10">
-        <f>IF($B57="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B57,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D57" s="13">
-        <f>IF($B57="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B57,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E57" s="10">
-        <f>IF($B57="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B57)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B57)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B57)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="12" t="n"/>
-      <c r="B58" s="10">
-        <f>IF($A58="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A58),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C58" s="10">
-        <f>IF($B58="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B58,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D58" s="13">
-        <f>IF($B58="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B58,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E58" s="10">
-        <f>IF($B58="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B58)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B58)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B58)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="12" t="n"/>
-      <c r="B59" s="10">
-        <f>IF($A59="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A59),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C59" s="10">
-        <f>IF($B59="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B59,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D59" s="13">
-        <f>IF($B59="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B59,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E59" s="10">
-        <f>IF($B59="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B59)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B59)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B59)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="12" t="n"/>
-      <c r="B60" s="10">
-        <f>IF($A60="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A60),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C60" s="10">
-        <f>IF($B60="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B60,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D60" s="13">
-        <f>IF($B60="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B60,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E60" s="10">
-        <f>IF($B60="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B60)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B60)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B60)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="12" t="n"/>
-      <c r="B61" s="10">
-        <f>IF($A61="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A61),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C61" s="10">
-        <f>IF($B61="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B61,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D61" s="13">
-        <f>IF($B61="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B61,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E61" s="10">
-        <f>IF($B61="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B61)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B61)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B61)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="12" t="n"/>
-      <c r="B62" s="10">
-        <f>IF($A62="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A62),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C62" s="10">
-        <f>IF($B62="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B62,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D62" s="13">
-        <f>IF($B62="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B62,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E62" s="10">
-        <f>IF($B62="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B62)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B62)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B62)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="12" t="n"/>
-      <c r="B63" s="10">
-        <f>IF($A63="","",TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER($A63),"ё","yo"),"ю","yu"),"я","ya"),"ц","ts"),"ч","ch"),"ш","sh"),"щ","sh"),"ў","o"),"қ","q"),"ғ","g"),"ҳ","h"),"а","a"),"б","b"),"в","v"),"г","g"),"д","d"),"е","e"),"ж","j"),"з","z"),"и","i"),"й","y"),"к","k"),"л","l"),"м","m"),"н","n"),"о","o"),"п","p"),"р","r"),"с","s"),"т","t"),"у","u"),"ф","f"),"х","x"),"ъ",""),"ы","i"),"ь",""),"э","e"),"'",""),"‘",""),"’",""),"ʻ",""),"ʼ",""),"`","")))</f>
-        <v/>
-      </c>
-      <c r="C63" s="10">
-        <f>IF($B63="","",IFERROR(INDEX('CRM Clients'!$A$4:$A$53,MATCH($B63,'CRM Clients'!$D$4:$D$53,0)),"not found"))</f>
-        <v/>
-      </c>
-      <c r="D63" s="13">
-        <f>IF($B63="","",IFERROR(INDEX('CRM Clients'!$B$4:$B$53,MATCH($B63,'CRM Clients'!$D$4:$D$53,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E63" s="10">
-        <f>IF($B63="","",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B63)=0,"no match - new client, or a typo",IF(COUNTIF('CRM Clients'!$D$4:$D$53,$B63)&gt;1,"CHECK PHONE - "&amp;COUNTIF('CRM Clients'!$D$4:$D$53,$B63)&amp;" clients share this name","matched")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Matching is exact after normalising, not fuzzy: it forgives alphabet and capitalisation, not misspellings. 'no match' on a name you expect usually means a real spelling difference - compare the Normalised column against the CRM Clients sheet.</t>
         </is>
@@ -3301,7 +3088,7 @@
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A46:E46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -3314,7 +3101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3842,156 +3629,6 @@
       </c>
       <c r="D33" s="10">
         <f>IF($C33="","",IF($C33="?","cannot read - fix by hand","ok"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="n"/>
-      <c r="B34" s="13">
-        <f>IF($A34="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($A34," ",""),"+",""),"-",""),"(",""),")",""),".",""),"/",""),CHAR(160),""))</f>
-        <v/>
-      </c>
-      <c r="C34" s="13">
-        <f>IF($B34="","",IF(AND(LEN($B34)=12,LEFT($B34,3)="998"),$B34,IF(LEN($B34)=9,"998"&amp;$B34,IF(AND(LEN($B34)=10,LEFT($B34,1)="8"),"998"&amp;MID($B34,2,9),IF(AND(LEN($B34)=14,LEFT($B34,5)="00998"),MID($B34,3,12),"?")))))</f>
-        <v/>
-      </c>
-      <c r="D34" s="10">
-        <f>IF($C34="","",IF($C34="?","cannot read - fix by hand","ok"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="n"/>
-      <c r="B35" s="13">
-        <f>IF($A35="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($A35," ",""),"+",""),"-",""),"(",""),")",""),".",""),"/",""),CHAR(160),""))</f>
-        <v/>
-      </c>
-      <c r="C35" s="13">
-        <f>IF($B35="","",IF(AND(LEN($B35)=12,LEFT($B35,3)="998"),$B35,IF(LEN($B35)=9,"998"&amp;$B35,IF(AND(LEN($B35)=10,LEFT($B35,1)="8"),"998"&amp;MID($B35,2,9),IF(AND(LEN($B35)=14,LEFT($B35,5)="00998"),MID($B35,3,12),"?")))))</f>
-        <v/>
-      </c>
-      <c r="D35" s="10">
-        <f>IF($C35="","",IF($C35="?","cannot read - fix by hand","ok"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="n"/>
-      <c r="B36" s="13">
-        <f>IF($A36="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($A36," ",""),"+",""),"-",""),"(",""),")",""),".",""),"/",""),CHAR(160),""))</f>
-        <v/>
-      </c>
-      <c r="C36" s="13">
-        <f>IF($B36="","",IF(AND(LEN($B36)=12,LEFT($B36,3)="998"),$B36,IF(LEN($B36)=9,"998"&amp;$B36,IF(AND(LEN($B36)=10,LEFT($B36,1)="8"),"998"&amp;MID($B36,2,9),IF(AND(LEN($B36)=14,LEFT($B36,5)="00998"),MID($B36,3,12),"?")))))</f>
-        <v/>
-      </c>
-      <c r="D36" s="10">
-        <f>IF($C36="","",IF($C36="?","cannot read - fix by hand","ok"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="12" t="n"/>
-      <c r="B37" s="13">
-        <f>IF($A37="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($A37," ",""),"+",""),"-",""),"(",""),")",""),".",""),"/",""),CHAR(160),""))</f>
-        <v/>
-      </c>
-      <c r="C37" s="13">
-        <f>IF($B37="","",IF(AND(LEN($B37)=12,LEFT($B37,3)="998"),$B37,IF(LEN($B37)=9,"998"&amp;$B37,IF(AND(LEN($B37)=10,LEFT($B37,1)="8"),"998"&amp;MID($B37,2,9),IF(AND(LEN($B37)=14,LEFT($B37,5)="00998"),MID($B37,3,12),"?")))))</f>
-        <v/>
-      </c>
-      <c r="D37" s="10">
-        <f>IF($C37="","",IF($C37="?","cannot read - fix by hand","ok"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="12" t="n"/>
-      <c r="B38" s="13">
-        <f>IF($A38="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($A38," ",""),"+",""),"-",""),"(",""),")",""),".",""),"/",""),CHAR(160),""))</f>
-        <v/>
-      </c>
-      <c r="C38" s="13">
-        <f>IF($B38="","",IF(AND(LEN($B38)=12,LEFT($B38,3)="998"),$B38,IF(LEN($B38)=9,"998"&amp;$B38,IF(AND(LEN($B38)=10,LEFT($B38,1)="8"),"998"&amp;MID($B38,2,9),IF(AND(LEN($B38)=14,LEFT($B38,5)="00998"),MID($B38,3,12),"?")))))</f>
-        <v/>
-      </c>
-      <c r="D38" s="10">
-        <f>IF($C38="","",IF($C38="?","cannot read - fix by hand","ok"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="12" t="n"/>
-      <c r="B39" s="13">
-        <f>IF($A39="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($A39," ",""),"+",""),"-",""),"(",""),")",""),".",""),"/",""),CHAR(160),""))</f>
-        <v/>
-      </c>
-      <c r="C39" s="13">
-        <f>IF($B39="","",IF(AND(LEN($B39)=12,LEFT($B39,3)="998"),$B39,IF(LEN($B39)=9,"998"&amp;$B39,IF(AND(LEN($B39)=10,LEFT($B39,1)="8"),"998"&amp;MID($B39,2,9),IF(AND(LEN($B39)=14,LEFT($B39,5)="00998"),MID($B39,3,12),"?")))))</f>
-        <v/>
-      </c>
-      <c r="D39" s="10">
-        <f>IF($C39="","",IF($C39="?","cannot read - fix by hand","ok"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="12" t="n"/>
-      <c r="B40" s="13">
-        <f>IF($A40="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($A40," ",""),"+",""),"-",""),"(",""),")",""),".",""),"/",""),CHAR(160),""))</f>
-        <v/>
-      </c>
-      <c r="C40" s="13">
-        <f>IF($B40="","",IF(AND(LEN($B40)=12,LEFT($B40,3)="998"),$B40,IF(LEN($B40)=9,"998"&amp;$B40,IF(AND(LEN($B40)=10,LEFT($B40,1)="8"),"998"&amp;MID($B40,2,9),IF(AND(LEN($B40)=14,LEFT($B40,5)="00998"),MID($B40,3,12),"?")))))</f>
-        <v/>
-      </c>
-      <c r="D40" s="10">
-        <f>IF($C40="","",IF($C40="?","cannot read - fix by hand","ok"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="12" t="n"/>
-      <c r="B41" s="13">
-        <f>IF($A41="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($A41," ",""),"+",""),"-",""),"(",""),")",""),".",""),"/",""),CHAR(160),""))</f>
-        <v/>
-      </c>
-      <c r="C41" s="13">
-        <f>IF($B41="","",IF(AND(LEN($B41)=12,LEFT($B41,3)="998"),$B41,IF(LEN($B41)=9,"998"&amp;$B41,IF(AND(LEN($B41)=10,LEFT($B41,1)="8"),"998"&amp;MID($B41,2,9),IF(AND(LEN($B41)=14,LEFT($B41,5)="00998"),MID($B41,3,12),"?")))))</f>
-        <v/>
-      </c>
-      <c r="D41" s="10">
-        <f>IF($C41="","",IF($C41="?","cannot read - fix by hand","ok"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="12" t="n"/>
-      <c r="B42" s="13">
-        <f>IF($A42="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($A42," ",""),"+",""),"-",""),"(",""),")",""),".",""),"/",""),CHAR(160),""))</f>
-        <v/>
-      </c>
-      <c r="C42" s="13">
-        <f>IF($B42="","",IF(AND(LEN($B42)=12,LEFT($B42,3)="998"),$B42,IF(LEN($B42)=9,"998"&amp;$B42,IF(AND(LEN($B42)=10,LEFT($B42,1)="8"),"998"&amp;MID($B42,2,9),IF(AND(LEN($B42)=14,LEFT($B42,5)="00998"),MID($B42,3,12),"?")))))</f>
-        <v/>
-      </c>
-      <c r="D42" s="10">
-        <f>IF($C42="","",IF($C42="?","cannot read - fix by hand","ok"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="12" t="n"/>
-      <c r="B43" s="13">
-        <f>IF($A43="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($A43," ",""),"+",""),"-",""),"(",""),")",""),".",""),"/",""),CHAR(160),""))</f>
-        <v/>
-      </c>
-      <c r="C43" s="13">
-        <f>IF($B43="","",IF(AND(LEN($B43)=12,LEFT($B43,3)="998"),$B43,IF(LEN($B43)=9,"998"&amp;$B43,IF(AND(LEN($B43)=10,LEFT($B43,1)="8"),"998"&amp;MID($B43,2,9),IF(AND(LEN($B43)=14,LEFT($B43,5)="00998"),MID($B43,3,12),"?")))))</f>
-        <v/>
-      </c>
-      <c r="D43" s="10">
-        <f>IF($C43="","",IF($C43="?","cannot read - fix by hand","ok"))</f>
         <v/>
       </c>
     </row>
@@ -4530,14 +4167,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="92" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -4565,7 +4210,12 @@
           <t>In words</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>working - the four digit groups, then their words</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>lookup tables - leave alone</t>
         </is>
@@ -4576,50 +4226,146 @@
         <v>13500000</v>
       </c>
       <c r="B4" s="10">
-        <f>IF($A4="","",IF(INT($A4)=0,"nol so'm",TRIM(IF(INT(INT($A4)/1000000000)&gt;0,IF(INT(INT($A4)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A4)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A4)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A4)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A4)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A4)/1000000000),100),10)+1),IF(MOD(INT(INT($A4)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A4)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A4)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A4),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A4),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A4),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A4),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A4),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A4),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A4),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A4),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A4),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A4),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A4),1000000)/1000)&gt;0,IF(INT(MOD(INT($A4),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A4),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A4),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A4),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A4),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A4),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A4),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A4),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A4),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A4),1000)=0,"",TRIM(IF(INT(MOD(INT($A4),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A4),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A4),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A4),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A4),1000),100),10)+1),IF(MOD(MOD(INT($A4),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A4),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A4),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-      <c r="H4" s="2" t="n">
+        <f>IF($A4="","",IF(INT($A4)=0,"nol so'm",TRIM(IF($D4&gt;0,$H4&amp;" milliard ","")&amp;IF($E4&gt;0,$I4&amp;" million ","")&amp;IF($F4&gt;0,$J4&amp;" ming ","")&amp;$K4)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D4" s="21">
+        <f>IF($A4="","",INT(INT($A4)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E4" s="21">
+        <f>IF($A4="","",INT(MOD(INT($A4),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F4" s="21">
+        <f>IF($A4="","",INT(MOD(INT($A4),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G4" s="21">
+        <f>IF($A4="","",MOD(INT($A4),1000))</f>
+        <v/>
+      </c>
+      <c r="H4" s="21">
+        <f>IF($A4="","",IF($D4=0,"",TRIM(IF(INT($D4/100)&gt;0,INDEX($N$4:$N$13,INT($D4/100)+1)&amp;" yuz ","")&amp;IF(MOD($D4,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D4,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D4,100),10)+1),IF(MOD($D4,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D4,100)-10+1),INDEX($N$4:$N$13,MOD($D4,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I4" s="21">
+        <f>IF($A4="","",IF($E4=0,"",TRIM(IF(INT($E4/100)&gt;0,INDEX($N$4:$N$13,INT($E4/100)+1)&amp;" yuz ","")&amp;IF(MOD($E4,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E4,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E4,100),10)+1),IF(MOD($E4,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E4,100)-10+1),INDEX($N$4:$N$13,MOD($E4,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J4" s="21">
+        <f>IF($A4="","",IF($F4=0,"",TRIM(IF(INT($F4/100)&gt;0,INDEX($N$4:$N$13,INT($F4/100)+1)&amp;" yuz ","")&amp;IF(MOD($F4,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F4,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F4,100),10)+1),IF(MOD($F4,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F4,100)-10+1),INDEX($N$4:$N$13,MOD($F4,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K4" s="21">
+        <f>IF($A4="","",IF($G4=0,"",TRIM(IF(INT($G4/100)&gt;0,INDEX($N$4:$N$13,INT($G4/100)+1)&amp;" yuz ","")&amp;IF(MOD($G4,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G4,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G4,100),10)+1),IF(MOD($G4,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G4,100)-10+1),INDEX($N$4:$N$13,MOD($G4,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="M4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>3005040</v>
       </c>
       <c r="B5" s="10">
-        <f>IF($A5="","",IF(INT($A5)=0,"nol so'm",TRIM(IF(INT(INT($A5)/1000000000)&gt;0,IF(INT(INT($A5)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A5)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A5)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A5)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A5)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A5)/1000000000),100),10)+1),IF(MOD(INT(INT($A5)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A5)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A5)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A5),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A5),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A5),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A5),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A5),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A5),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A5),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A5),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A5),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A5),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A5),1000000)/1000)&gt;0,IF(INT(MOD(INT($A5),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A5),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A5),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A5),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A5),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A5),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A5),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A5),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A5),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A5),1000)=0,"",TRIM(IF(INT(MOD(INT($A5),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A5),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A5),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A5),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A5),1000),100),10)+1),IF(MOD(MOD(INT($A5),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A5),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A5),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-      <c r="H5" s="2" t="n">
+        <f>IF($A5="","",IF(INT($A5)=0,"nol so'm",TRIM(IF($D5&gt;0,$H5&amp;" milliard ","")&amp;IF($E5&gt;0,$I5&amp;" million ","")&amp;IF($F5&gt;0,$J5&amp;" ming ","")&amp;$K5)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D5" s="21">
+        <f>IF($A5="","",INT(INT($A5)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E5" s="21">
+        <f>IF($A5="","",INT(MOD(INT($A5),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F5" s="21">
+        <f>IF($A5="","",INT(MOD(INT($A5),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G5" s="21">
+        <f>IF($A5="","",MOD(INT($A5),1000))</f>
+        <v/>
+      </c>
+      <c r="H5" s="21">
+        <f>IF($A5="","",IF($D5=0,"",TRIM(IF(INT($D5/100)&gt;0,INDEX($N$4:$N$13,INT($D5/100)+1)&amp;" yuz ","")&amp;IF(MOD($D5,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D5,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D5,100),10)+1),IF(MOD($D5,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D5,100)-10+1),INDEX($N$4:$N$13,MOD($D5,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I5" s="21">
+        <f>IF($A5="","",IF($E5=0,"",TRIM(IF(INT($E5/100)&gt;0,INDEX($N$4:$N$13,INT($E5/100)+1)&amp;" yuz ","")&amp;IF(MOD($E5,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E5,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E5,100),10)+1),IF(MOD($E5,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E5,100)-10+1),INDEX($N$4:$N$13,MOD($E5,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J5" s="21">
+        <f>IF($A5="","",IF($F5=0,"",TRIM(IF(INT($F5/100)&gt;0,INDEX($N$4:$N$13,INT($F5/100)+1)&amp;" yuz ","")&amp;IF(MOD($F5,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F5,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F5,100),10)+1),IF(MOD($F5,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F5,100)-10+1),INDEX($N$4:$N$13,MOD($F5,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K5" s="21">
+        <f>IF($A5="","",IF($G5=0,"",TRIM(IF(INT($G5/100)&gt;0,INDEX($N$4:$N$13,INT($G5/100)+1)&amp;" yuz ","")&amp;IF(MOD($G5,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G5,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G5,100),10)+1),IF(MOD($G5,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G5,100)-10+1),INDEX($N$4:$N$13,MOD($G5,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="M5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>bir</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>22500000</v>
       </c>
       <c r="B6" s="10">
-        <f>IF($A6="","",IF(INT($A6)=0,"nol so'm",TRIM(IF(INT(INT($A6)/1000000000)&gt;0,IF(INT(INT($A6)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A6)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A6)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A6)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A6)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A6)/1000000000),100),10)+1),IF(MOD(INT(INT($A6)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A6)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A6)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A6),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A6),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A6),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A6),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A6),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A6),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A6),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A6),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A6),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A6),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A6),1000000)/1000)&gt;0,IF(INT(MOD(INT($A6),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A6),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A6),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A6),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A6),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A6),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A6),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A6),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A6),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A6),1000)=0,"",TRIM(IF(INT(MOD(INT($A6),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A6),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A6),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A6),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A6),1000),100),10)+1),IF(MOD(MOD(INT($A6),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A6),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A6),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-      <c r="H6" s="2" t="n">
+        <f>IF($A6="","",IF(INT($A6)=0,"nol so'm",TRIM(IF($D6&gt;0,$H6&amp;" milliard ","")&amp;IF($E6&gt;0,$I6&amp;" million ","")&amp;IF($F6&gt;0,$J6&amp;" ming ","")&amp;$K6)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D6" s="21">
+        <f>IF($A6="","",INT(INT($A6)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E6" s="21">
+        <f>IF($A6="","",INT(MOD(INT($A6),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F6" s="21">
+        <f>IF($A6="","",INT(MOD(INT($A6),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G6" s="21">
+        <f>IF($A6="","",MOD(INT($A6),1000))</f>
+        <v/>
+      </c>
+      <c r="H6" s="21">
+        <f>IF($A6="","",IF($D6=0,"",TRIM(IF(INT($D6/100)&gt;0,INDEX($N$4:$N$13,INT($D6/100)+1)&amp;" yuz ","")&amp;IF(MOD($D6,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D6,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D6,100),10)+1),IF(MOD($D6,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D6,100)-10+1),INDEX($N$4:$N$13,MOD($D6,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I6" s="21">
+        <f>IF($A6="","",IF($E6=0,"",TRIM(IF(INT($E6/100)&gt;0,INDEX($N$4:$N$13,INT($E6/100)+1)&amp;" yuz ","")&amp;IF(MOD($E6,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E6,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E6,100),10)+1),IF(MOD($E6,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E6,100)-10+1),INDEX($N$4:$N$13,MOD($E6,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J6" s="21">
+        <f>IF($A6="","",IF($F6=0,"",TRIM(IF(INT($F6/100)&gt;0,INDEX($N$4:$N$13,INT($F6/100)+1)&amp;" yuz ","")&amp;IF(MOD($F6,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F6,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F6,100),10)+1),IF(MOD($F6,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F6,100)-10+1),INDEX($N$4:$N$13,MOD($F6,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K6" s="21">
+        <f>IF($A6="","",IF($G6=0,"",TRIM(IF(INT($G6/100)&gt;0,INDEX($N$4:$N$13,INT($G6/100)+1)&amp;" yuz ","")&amp;IF(MOD($G6,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G6,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G6,100),10)+1),IF(MOD($G6,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G6,100)-10+1),INDEX($N$4:$N$13,MOD($G6,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="M6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>ikki</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>yigirma</t>
         </is>
@@ -4630,18 +4376,50 @@
         <v>245508000</v>
       </c>
       <c r="B7" s="10">
-        <f>IF($A7="","",IF(INT($A7)=0,"nol so'm",TRIM(IF(INT(INT($A7)/1000000000)&gt;0,IF(INT(INT($A7)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A7)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A7)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A7)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A7)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A7)/1000000000),100),10)+1),IF(MOD(INT(INT($A7)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A7)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A7)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A7),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A7),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A7),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A7),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A7),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A7),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A7),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A7),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A7),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A7),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A7),1000000)/1000)&gt;0,IF(INT(MOD(INT($A7),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A7),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A7),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A7),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A7),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A7),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A7),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A7),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A7),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A7),1000)=0,"",TRIM(IF(INT(MOD(INT($A7),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A7),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A7),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A7),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A7),1000),100),10)+1),IF(MOD(MOD(INT($A7),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A7),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A7),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-      <c r="H7" s="2" t="n">
+        <f>IF($A7="","",IF(INT($A7)=0,"nol so'm",TRIM(IF($D7&gt;0,$H7&amp;" milliard ","")&amp;IF($E7&gt;0,$I7&amp;" million ","")&amp;IF($F7&gt;0,$J7&amp;" ming ","")&amp;$K7)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D7" s="21">
+        <f>IF($A7="","",INT(INT($A7)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E7" s="21">
+        <f>IF($A7="","",INT(MOD(INT($A7),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F7" s="21">
+        <f>IF($A7="","",INT(MOD(INT($A7),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G7" s="21">
+        <f>IF($A7="","",MOD(INT($A7),1000))</f>
+        <v/>
+      </c>
+      <c r="H7" s="21">
+        <f>IF($A7="","",IF($D7=0,"",TRIM(IF(INT($D7/100)&gt;0,INDEX($N$4:$N$13,INT($D7/100)+1)&amp;" yuz ","")&amp;IF(MOD($D7,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D7,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D7,100),10)+1),IF(MOD($D7,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D7,100)-10+1),INDEX($N$4:$N$13,MOD($D7,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I7" s="21">
+        <f>IF($A7="","",IF($E7=0,"",TRIM(IF(INT($E7/100)&gt;0,INDEX($N$4:$N$13,INT($E7/100)+1)&amp;" yuz ","")&amp;IF(MOD($E7,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E7,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E7,100),10)+1),IF(MOD($E7,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E7,100)-10+1),INDEX($N$4:$N$13,MOD($E7,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J7" s="21">
+        <f>IF($A7="","",IF($F7=0,"",TRIM(IF(INT($F7/100)&gt;0,INDEX($N$4:$N$13,INT($F7/100)+1)&amp;" yuz ","")&amp;IF(MOD($F7,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F7,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F7,100),10)+1),IF(MOD($F7,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F7,100)-10+1),INDEX($N$4:$N$13,MOD($F7,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K7" s="21">
+        <f>IF($A7="","",IF($G7=0,"",TRIM(IF(INT($G7/100)&gt;0,INDEX($N$4:$N$13,INT($G7/100)+1)&amp;" yuz ","")&amp;IF(MOD($G7,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G7,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G7,100),10)+1),IF(MOD($G7,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G7,100)-10+1),INDEX($N$4:$N$13,MOD($G7,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="M7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>uch</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>o'ttiz</t>
         </is>
@@ -4652,18 +4430,50 @@
         <v>1500</v>
       </c>
       <c r="B8" s="10">
-        <f>IF($A8="","",IF(INT($A8)=0,"nol so'm",TRIM(IF(INT(INT($A8)/1000000000)&gt;0,IF(INT(INT($A8)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A8)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A8)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A8)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A8)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A8)/1000000000),100),10)+1),IF(MOD(INT(INT($A8)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A8)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A8)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A8),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A8),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A8),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A8),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A8),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A8),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A8),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A8),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A8),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A8),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A8),1000000)/1000)&gt;0,IF(INT(MOD(INT($A8),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A8),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A8),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A8),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A8),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A8),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A8),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A8),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A8),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A8),1000)=0,"",TRIM(IF(INT(MOD(INT($A8),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A8),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A8),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A8),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A8),1000),100),10)+1),IF(MOD(MOD(INT($A8),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A8),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A8),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-      <c r="H8" s="2" t="n">
+        <f>IF($A8="","",IF(INT($A8)=0,"nol so'm",TRIM(IF($D8&gt;0,$H8&amp;" milliard ","")&amp;IF($E8&gt;0,$I8&amp;" million ","")&amp;IF($F8&gt;0,$J8&amp;" ming ","")&amp;$K8)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D8" s="21">
+        <f>IF($A8="","",INT(INT($A8)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E8" s="21">
+        <f>IF($A8="","",INT(MOD(INT($A8),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F8" s="21">
+        <f>IF($A8="","",INT(MOD(INT($A8),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G8" s="21">
+        <f>IF($A8="","",MOD(INT($A8),1000))</f>
+        <v/>
+      </c>
+      <c r="H8" s="21">
+        <f>IF($A8="","",IF($D8=0,"",TRIM(IF(INT($D8/100)&gt;0,INDEX($N$4:$N$13,INT($D8/100)+1)&amp;" yuz ","")&amp;IF(MOD($D8,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D8,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D8,100),10)+1),IF(MOD($D8,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D8,100)-10+1),INDEX($N$4:$N$13,MOD($D8,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I8" s="21">
+        <f>IF($A8="","",IF($E8=0,"",TRIM(IF(INT($E8/100)&gt;0,INDEX($N$4:$N$13,INT($E8/100)+1)&amp;" yuz ","")&amp;IF(MOD($E8,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E8,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E8,100),10)+1),IF(MOD($E8,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E8,100)-10+1),INDEX($N$4:$N$13,MOD($E8,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J8" s="21">
+        <f>IF($A8="","",IF($F8=0,"",TRIM(IF(INT($F8/100)&gt;0,INDEX($N$4:$N$13,INT($F8/100)+1)&amp;" yuz ","")&amp;IF(MOD($F8,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F8,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F8,100),10)+1),IF(MOD($F8,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F8,100)-10+1),INDEX($N$4:$N$13,MOD($F8,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K8" s="21">
+        <f>IF($A8="","",IF($G8=0,"",TRIM(IF(INT($G8/100)&gt;0,INDEX($N$4:$N$13,INT($G8/100)+1)&amp;" yuz ","")&amp;IF(MOD($G8,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G8,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G8,100),10)+1),IF(MOD($G8,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G8,100)-10+1),INDEX($N$4:$N$13,MOD($G8,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="M8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>to'rt</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>qirq</t>
         </is>
@@ -4674,18 +4484,50 @@
         <v>9262000</v>
       </c>
       <c r="B9" s="10">
-        <f>IF($A9="","",IF(INT($A9)=0,"nol so'm",TRIM(IF(INT(INT($A9)/1000000000)&gt;0,IF(INT(INT($A9)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A9)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A9)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A9)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A9)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A9)/1000000000),100),10)+1),IF(MOD(INT(INT($A9)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A9)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A9)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A9),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A9),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A9),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A9),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A9),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A9),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A9),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A9),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A9),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A9),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A9),1000000)/1000)&gt;0,IF(INT(MOD(INT($A9),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A9),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A9),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A9),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A9),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A9),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A9),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A9),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A9),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A9),1000)=0,"",TRIM(IF(INT(MOD(INT($A9),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A9),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A9),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A9),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A9),1000),100),10)+1),IF(MOD(MOD(INT($A9),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A9),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A9),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-      <c r="H9" s="2" t="n">
+        <f>IF($A9="","",IF(INT($A9)=0,"nol so'm",TRIM(IF($D9&gt;0,$H9&amp;" milliard ","")&amp;IF($E9&gt;0,$I9&amp;" million ","")&amp;IF($F9&gt;0,$J9&amp;" ming ","")&amp;$K9)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D9" s="21">
+        <f>IF($A9="","",INT(INT($A9)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E9" s="21">
+        <f>IF($A9="","",INT(MOD(INT($A9),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F9" s="21">
+        <f>IF($A9="","",INT(MOD(INT($A9),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G9" s="21">
+        <f>IF($A9="","",MOD(INT($A9),1000))</f>
+        <v/>
+      </c>
+      <c r="H9" s="21">
+        <f>IF($A9="","",IF($D9=0,"",TRIM(IF(INT($D9/100)&gt;0,INDEX($N$4:$N$13,INT($D9/100)+1)&amp;" yuz ","")&amp;IF(MOD($D9,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D9,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D9,100),10)+1),IF(MOD($D9,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D9,100)-10+1),INDEX($N$4:$N$13,MOD($D9,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I9" s="21">
+        <f>IF($A9="","",IF($E9=0,"",TRIM(IF(INT($E9/100)&gt;0,INDEX($N$4:$N$13,INT($E9/100)+1)&amp;" yuz ","")&amp;IF(MOD($E9,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E9,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E9,100),10)+1),IF(MOD($E9,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E9,100)-10+1),INDEX($N$4:$N$13,MOD($E9,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J9" s="21">
+        <f>IF($A9="","",IF($F9=0,"",TRIM(IF(INT($F9/100)&gt;0,INDEX($N$4:$N$13,INT($F9/100)+1)&amp;" yuz ","")&amp;IF(MOD($F9,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F9,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F9,100),10)+1),IF(MOD($F9,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F9,100)-10+1),INDEX($N$4:$N$13,MOD($F9,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K9" s="21">
+        <f>IF($A9="","",IF($G9=0,"",TRIM(IF(INT($G9/100)&gt;0,INDEX($N$4:$N$13,INT($G9/100)+1)&amp;" yuz ","")&amp;IF(MOD($G9,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G9,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G9,100),10)+1),IF(MOD($G9,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G9,100)-10+1),INDEX($N$4:$N$13,MOD($G9,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="M9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>besh</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>ellik</t>
         </is>
@@ -4694,18 +4536,50 @@
     <row r="10">
       <c r="A10" s="20" t="n"/>
       <c r="B10" s="10">
-        <f>IF($A10="","",IF(INT($A10)=0,"nol so'm",TRIM(IF(INT(INT($A10)/1000000000)&gt;0,IF(INT(INT($A10)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A10)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A10)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A10)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A10)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A10)/1000000000),100),10)+1),IF(MOD(INT(INT($A10)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A10)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A10)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A10),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A10),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A10),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A10),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A10),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A10),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A10),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A10),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A10),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A10),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A10),1000000)/1000)&gt;0,IF(INT(MOD(INT($A10),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A10),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A10),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A10),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A10),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A10),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A10),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A10),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A10),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A10),1000)=0,"",TRIM(IF(INT(MOD(INT($A10),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A10),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A10),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A10),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A10),1000),100),10)+1),IF(MOD(MOD(INT($A10),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A10),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A10),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-      <c r="H10" s="2" t="n">
+        <f>IF($A10="","",IF(INT($A10)=0,"nol so'm",TRIM(IF($D10&gt;0,$H10&amp;" milliard ","")&amp;IF($E10&gt;0,$I10&amp;" million ","")&amp;IF($F10&gt;0,$J10&amp;" ming ","")&amp;$K10)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D10" s="21">
+        <f>IF($A10="","",INT(INT($A10)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>IF($A10="","",INT(MOD(INT($A10),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>IF($A10="","",INT(MOD(INT($A10),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>IF($A10="","",MOD(INT($A10),1000))</f>
+        <v/>
+      </c>
+      <c r="H10" s="21">
+        <f>IF($A10="","",IF($D10=0,"",TRIM(IF(INT($D10/100)&gt;0,INDEX($N$4:$N$13,INT($D10/100)+1)&amp;" yuz ","")&amp;IF(MOD($D10,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D10,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D10,100),10)+1),IF(MOD($D10,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D10,100)-10+1),INDEX($N$4:$N$13,MOD($D10,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I10" s="21">
+        <f>IF($A10="","",IF($E10=0,"",TRIM(IF(INT($E10/100)&gt;0,INDEX($N$4:$N$13,INT($E10/100)+1)&amp;" yuz ","")&amp;IF(MOD($E10,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E10,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E10,100),10)+1),IF(MOD($E10,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E10,100)-10+1),INDEX($N$4:$N$13,MOD($E10,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J10" s="21">
+        <f>IF($A10="","",IF($F10=0,"",TRIM(IF(INT($F10/100)&gt;0,INDEX($N$4:$N$13,INT($F10/100)+1)&amp;" yuz ","")&amp;IF(MOD($F10,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F10,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F10,100),10)+1),IF(MOD($F10,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F10,100)-10+1),INDEX($N$4:$N$13,MOD($F10,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K10" s="21">
+        <f>IF($A10="","",IF($G10=0,"",TRIM(IF(INT($G10/100)&gt;0,INDEX($N$4:$N$13,INT($G10/100)+1)&amp;" yuz ","")&amp;IF(MOD($G10,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G10,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G10,100),10)+1),IF(MOD($G10,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G10,100)-10+1),INDEX($N$4:$N$13,MOD($G10,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="M10" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>olti</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>oltmish</t>
         </is>
@@ -4714,18 +4588,50 @@
     <row r="11">
       <c r="A11" s="20" t="n"/>
       <c r="B11" s="10">
-        <f>IF($A11="","",IF(INT($A11)=0,"nol so'm",TRIM(IF(INT(INT($A11)/1000000000)&gt;0,IF(INT(INT($A11)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A11)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A11)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A11)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A11)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A11)/1000000000),100),10)+1),IF(MOD(INT(INT($A11)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A11)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A11)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A11),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A11),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A11),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A11),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A11),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A11),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A11),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A11),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A11),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A11),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A11),1000000)/1000)&gt;0,IF(INT(MOD(INT($A11),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A11),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A11),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A11),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A11),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A11),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A11),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A11),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A11),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A11),1000)=0,"",TRIM(IF(INT(MOD(INT($A11),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A11),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A11),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A11),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A11),1000),100),10)+1),IF(MOD(MOD(INT($A11),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A11),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A11),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-      <c r="H11" s="2" t="n">
+        <f>IF($A11="","",IF(INT($A11)=0,"nol so'm",TRIM(IF($D11&gt;0,$H11&amp;" milliard ","")&amp;IF($E11&gt;0,$I11&amp;" million ","")&amp;IF($F11&gt;0,$J11&amp;" ming ","")&amp;$K11)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D11" s="21">
+        <f>IF($A11="","",INT(INT($A11)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E11" s="21">
+        <f>IF($A11="","",INT(MOD(INT($A11),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F11" s="21">
+        <f>IF($A11="","",INT(MOD(INT($A11),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G11" s="21">
+        <f>IF($A11="","",MOD(INT($A11),1000))</f>
+        <v/>
+      </c>
+      <c r="H11" s="21">
+        <f>IF($A11="","",IF($D11=0,"",TRIM(IF(INT($D11/100)&gt;0,INDEX($N$4:$N$13,INT($D11/100)+1)&amp;" yuz ","")&amp;IF(MOD($D11,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D11,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D11,100),10)+1),IF(MOD($D11,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D11,100)-10+1),INDEX($N$4:$N$13,MOD($D11,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I11" s="21">
+        <f>IF($A11="","",IF($E11=0,"",TRIM(IF(INT($E11/100)&gt;0,INDEX($N$4:$N$13,INT($E11/100)+1)&amp;" yuz ","")&amp;IF(MOD($E11,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E11,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E11,100),10)+1),IF(MOD($E11,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E11,100)-10+1),INDEX($N$4:$N$13,MOD($E11,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J11" s="21">
+        <f>IF($A11="","",IF($F11=0,"",TRIM(IF(INT($F11/100)&gt;0,INDEX($N$4:$N$13,INT($F11/100)+1)&amp;" yuz ","")&amp;IF(MOD($F11,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F11,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F11,100),10)+1),IF(MOD($F11,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F11,100)-10+1),INDEX($N$4:$N$13,MOD($F11,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K11" s="21">
+        <f>IF($A11="","",IF($G11=0,"",TRIM(IF(INT($G11/100)&gt;0,INDEX($N$4:$N$13,INT($G11/100)+1)&amp;" yuz ","")&amp;IF(MOD($G11,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G11,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G11,100),10)+1),IF(MOD($G11,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G11,100)-10+1),INDEX($N$4:$N$13,MOD($G11,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="M11" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>yetti</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>yetmish</t>
         </is>
@@ -4734,18 +4640,50 @@
     <row r="12">
       <c r="A12" s="20" t="n"/>
       <c r="B12" s="10">
-        <f>IF($A12="","",IF(INT($A12)=0,"nol so'm",TRIM(IF(INT(INT($A12)/1000000000)&gt;0,IF(INT(INT($A12)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A12)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A12)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A12)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A12)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A12)/1000000000),100),10)+1),IF(MOD(INT(INT($A12)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A12)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A12)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A12),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A12),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A12),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A12),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A12),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A12),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A12),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A12),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A12),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A12),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A12),1000000)/1000)&gt;0,IF(INT(MOD(INT($A12),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A12),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A12),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A12),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A12),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A12),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A12),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A12),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A12),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A12),1000)=0,"",TRIM(IF(INT(MOD(INT($A12),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A12),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A12),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A12),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A12),1000),100),10)+1),IF(MOD(MOD(INT($A12),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A12),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A12),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-      <c r="H12" s="2" t="n">
+        <f>IF($A12="","",IF(INT($A12)=0,"nol so'm",TRIM(IF($D12&gt;0,$H12&amp;" milliard ","")&amp;IF($E12&gt;0,$I12&amp;" million ","")&amp;IF($F12&gt;0,$J12&amp;" ming ","")&amp;$K12)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D12" s="21">
+        <f>IF($A12="","",INT(INT($A12)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E12" s="21">
+        <f>IF($A12="","",INT(MOD(INT($A12),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F12" s="21">
+        <f>IF($A12="","",INT(MOD(INT($A12),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G12" s="21">
+        <f>IF($A12="","",MOD(INT($A12),1000))</f>
+        <v/>
+      </c>
+      <c r="H12" s="21">
+        <f>IF($A12="","",IF($D12=0,"",TRIM(IF(INT($D12/100)&gt;0,INDEX($N$4:$N$13,INT($D12/100)+1)&amp;" yuz ","")&amp;IF(MOD($D12,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D12,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D12,100),10)+1),IF(MOD($D12,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D12,100)-10+1),INDEX($N$4:$N$13,MOD($D12,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I12" s="21">
+        <f>IF($A12="","",IF($E12=0,"",TRIM(IF(INT($E12/100)&gt;0,INDEX($N$4:$N$13,INT($E12/100)+1)&amp;" yuz ","")&amp;IF(MOD($E12,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E12,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E12,100),10)+1),IF(MOD($E12,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E12,100)-10+1),INDEX($N$4:$N$13,MOD($E12,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J12" s="21">
+        <f>IF($A12="","",IF($F12=0,"",TRIM(IF(INT($F12/100)&gt;0,INDEX($N$4:$N$13,INT($F12/100)+1)&amp;" yuz ","")&amp;IF(MOD($F12,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F12,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F12,100),10)+1),IF(MOD($F12,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F12,100)-10+1),INDEX($N$4:$N$13,MOD($F12,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K12" s="21">
+        <f>IF($A12="","",IF($G12=0,"",TRIM(IF(INT($G12/100)&gt;0,INDEX($N$4:$N$13,INT($G12/100)+1)&amp;" yuz ","")&amp;IF(MOD($G12,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G12,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G12,100),10)+1),IF(MOD($G12,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G12,100)-10+1),INDEX($N$4:$N$13,MOD($G12,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="M12" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>sakkiz</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>sakson</t>
         </is>
@@ -4754,18 +4692,50 @@
     <row r="13">
       <c r="A13" s="20" t="n"/>
       <c r="B13" s="10">
-        <f>IF($A13="","",IF(INT($A13)=0,"nol so'm",TRIM(IF(INT(INT($A13)/1000000000)&gt;0,IF(INT(INT($A13)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A13)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A13)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A13)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A13)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A13)/1000000000),100),10)+1),IF(MOD(INT(INT($A13)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A13)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A13)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A13),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A13),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A13),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A13),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A13),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A13),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A13),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A13),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A13),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A13),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A13),1000000)/1000)&gt;0,IF(INT(MOD(INT($A13),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A13),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A13),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A13),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A13),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A13),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A13),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A13),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A13),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A13),1000)=0,"",TRIM(IF(INT(MOD(INT($A13),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A13),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A13),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A13),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A13),1000),100),10)+1),IF(MOD(MOD(INT($A13),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A13),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A13),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-      <c r="H13" s="2" t="n">
+        <f>IF($A13="","",IF(INT($A13)=0,"nol so'm",TRIM(IF($D13&gt;0,$H13&amp;" milliard ","")&amp;IF($E13&gt;0,$I13&amp;" million ","")&amp;IF($F13&gt;0,$J13&amp;" ming ","")&amp;$K13)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D13" s="21">
+        <f>IF($A13="","",INT(INT($A13)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E13" s="21">
+        <f>IF($A13="","",INT(MOD(INT($A13),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F13" s="21">
+        <f>IF($A13="","",INT(MOD(INT($A13),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G13" s="21">
+        <f>IF($A13="","",MOD(INT($A13),1000))</f>
+        <v/>
+      </c>
+      <c r="H13" s="21">
+        <f>IF($A13="","",IF($D13=0,"",TRIM(IF(INT($D13/100)&gt;0,INDEX($N$4:$N$13,INT($D13/100)+1)&amp;" yuz ","")&amp;IF(MOD($D13,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D13,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D13,100),10)+1),IF(MOD($D13,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D13,100)-10+1),INDEX($N$4:$N$13,MOD($D13,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I13" s="21">
+        <f>IF($A13="","",IF($E13=0,"",TRIM(IF(INT($E13/100)&gt;0,INDEX($N$4:$N$13,INT($E13/100)+1)&amp;" yuz ","")&amp;IF(MOD($E13,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E13,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E13,100),10)+1),IF(MOD($E13,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E13,100)-10+1),INDEX($N$4:$N$13,MOD($E13,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J13" s="21">
+        <f>IF($A13="","",IF($F13=0,"",TRIM(IF(INT($F13/100)&gt;0,INDEX($N$4:$N$13,INT($F13/100)+1)&amp;" yuz ","")&amp;IF(MOD($F13,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F13,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F13,100),10)+1),IF(MOD($F13,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F13,100)-10+1),INDEX($N$4:$N$13,MOD($F13,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K13" s="21">
+        <f>IF($A13="","",IF($G13=0,"",TRIM(IF(INT($G13/100)&gt;0,INDEX($N$4:$N$13,INT($G13/100)+1)&amp;" yuz ","")&amp;IF(MOD($G13,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G13,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G13,100),10)+1),IF(MOD($G13,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G13,100)-10+1),INDEX($N$4:$N$13,MOD($G13,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="M13" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>to'qqiz</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>to'qson</t>
         </is>
@@ -4774,111 +4744,397 @@
     <row r="14">
       <c r="A14" s="20" t="n"/>
       <c r="B14" s="10">
-        <f>IF($A14="","",IF(INT($A14)=0,"nol so'm",TRIM(IF(INT(INT($A14)/1000000000)&gt;0,IF(INT(INT($A14)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A14)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A14)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A14)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A14)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A14)/1000000000),100),10)+1),IF(MOD(INT(INT($A14)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A14)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A14)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A14),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A14),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A14),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A14),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A14),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A14),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A14),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A14),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A14),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A14),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A14),1000000)/1000)&gt;0,IF(INT(MOD(INT($A14),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A14),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A14),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A14),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A14),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A14),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A14),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A14),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A14),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A14),1000)=0,"",TRIM(IF(INT(MOD(INT($A14),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A14),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A14),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A14),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A14),1000),100),10)+1),IF(MOD(MOD(INT($A14),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A14),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A14),1000),100)+1))))))&amp;" so'm"))</f>
+        <f>IF($A14="","",IF(INT($A14)=0,"nol so'm",TRIM(IF($D14&gt;0,$H14&amp;" milliard ","")&amp;IF($E14&gt;0,$I14&amp;" million ","")&amp;IF($F14&gt;0,$J14&amp;" ming ","")&amp;$K14)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D14" s="21">
+        <f>IF($A14="","",INT(INT($A14)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E14" s="21">
+        <f>IF($A14="","",INT(MOD(INT($A14),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F14" s="21">
+        <f>IF($A14="","",INT(MOD(INT($A14),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>IF($A14="","",MOD(INT($A14),1000))</f>
+        <v/>
+      </c>
+      <c r="H14" s="21">
+        <f>IF($A14="","",IF($D14=0,"",TRIM(IF(INT($D14/100)&gt;0,INDEX($N$4:$N$13,INT($D14/100)+1)&amp;" yuz ","")&amp;IF(MOD($D14,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D14,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D14,100),10)+1),IF(MOD($D14,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D14,100)-10+1),INDEX($N$4:$N$13,MOD($D14,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I14" s="21">
+        <f>IF($A14="","",IF($E14=0,"",TRIM(IF(INT($E14/100)&gt;0,INDEX($N$4:$N$13,INT($E14/100)+1)&amp;" yuz ","")&amp;IF(MOD($E14,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E14,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E14,100),10)+1),IF(MOD($E14,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E14,100)-10+1),INDEX($N$4:$N$13,MOD($E14,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J14" s="21">
+        <f>IF($A14="","",IF($F14=0,"",TRIM(IF(INT($F14/100)&gt;0,INDEX($N$4:$N$13,INT($F14/100)+1)&amp;" yuz ","")&amp;IF(MOD($F14,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F14,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F14,100),10)+1),IF(MOD($F14,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F14,100)-10+1),INDEX($N$4:$N$13,MOD($F14,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K14" s="21">
+        <f>IF($A14="","",IF($G14=0,"",TRIM(IF(INT($G14/100)&gt;0,INDEX($N$4:$N$13,INT($G14/100)+1)&amp;" yuz ","")&amp;IF(MOD($G14,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G14,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G14,100),10)+1),IF(MOD($G14,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G14,100)-10+1),INDEX($N$4:$N$13,MOD($G14,100)+1))))))</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n"/>
       <c r="B15" s="10">
-        <f>IF($A15="","",IF(INT($A15)=0,"nol so'm",TRIM(IF(INT(INT($A15)/1000000000)&gt;0,IF(INT(INT($A15)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A15)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A15)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A15)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A15)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A15)/1000000000),100),10)+1),IF(MOD(INT(INT($A15)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A15)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A15)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A15),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A15),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A15),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A15),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A15),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A15),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A15),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A15),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A15),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A15),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A15),1000000)/1000)&gt;0,IF(INT(MOD(INT($A15),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A15),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A15),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A15),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A15),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A15),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A15),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A15),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A15),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A15),1000)=0,"",TRIM(IF(INT(MOD(INT($A15),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A15),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A15),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A15),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A15),1000),100),10)+1),IF(MOD(MOD(INT($A15),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A15),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A15),1000),100)+1))))))&amp;" so'm"))</f>
+        <f>IF($A15="","",IF(INT($A15)=0,"nol so'm",TRIM(IF($D15&gt;0,$H15&amp;" milliard ","")&amp;IF($E15&gt;0,$I15&amp;" million ","")&amp;IF($F15&gt;0,$J15&amp;" ming ","")&amp;$K15)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D15" s="21">
+        <f>IF($A15="","",INT(INT($A15)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E15" s="21">
+        <f>IF($A15="","",INT(MOD(INT($A15),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F15" s="21">
+        <f>IF($A15="","",INT(MOD(INT($A15),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G15" s="21">
+        <f>IF($A15="","",MOD(INT($A15),1000))</f>
+        <v/>
+      </c>
+      <c r="H15" s="21">
+        <f>IF($A15="","",IF($D15=0,"",TRIM(IF(INT($D15/100)&gt;0,INDEX($N$4:$N$13,INT($D15/100)+1)&amp;" yuz ","")&amp;IF(MOD($D15,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D15,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D15,100),10)+1),IF(MOD($D15,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D15,100)-10+1),INDEX($N$4:$N$13,MOD($D15,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I15" s="21">
+        <f>IF($A15="","",IF($E15=0,"",TRIM(IF(INT($E15/100)&gt;0,INDEX($N$4:$N$13,INT($E15/100)+1)&amp;" yuz ","")&amp;IF(MOD($E15,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E15,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E15,100),10)+1),IF(MOD($E15,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E15,100)-10+1),INDEX($N$4:$N$13,MOD($E15,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J15" s="21">
+        <f>IF($A15="","",IF($F15=0,"",TRIM(IF(INT($F15/100)&gt;0,INDEX($N$4:$N$13,INT($F15/100)+1)&amp;" yuz ","")&amp;IF(MOD($F15,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F15,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F15,100),10)+1),IF(MOD($F15,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F15,100)-10+1),INDEX($N$4:$N$13,MOD($F15,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K15" s="21">
+        <f>IF($A15="","",IF($G15=0,"",TRIM(IF(INT($G15/100)&gt;0,INDEX($N$4:$N$13,INT($G15/100)+1)&amp;" yuz ","")&amp;IF(MOD($G15,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G15,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G15,100),10)+1),IF(MOD($G15,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G15,100)-10+1),INDEX($N$4:$N$13,MOD($G15,100)+1))))))</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n"/>
       <c r="B16" s="10">
-        <f>IF($A16="","",IF(INT($A16)=0,"nol so'm",TRIM(IF(INT(INT($A16)/1000000000)&gt;0,IF(INT(INT($A16)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A16)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A16)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A16)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A16)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A16)/1000000000),100),10)+1),IF(MOD(INT(INT($A16)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A16)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A16)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A16),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A16),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A16),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A16),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A16),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A16),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A16),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A16),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A16),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A16),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A16),1000000)/1000)&gt;0,IF(INT(MOD(INT($A16),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A16),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A16),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A16),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A16),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A16),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A16),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A16),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A16),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A16),1000)=0,"",TRIM(IF(INT(MOD(INT($A16),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A16),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A16),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A16),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A16),1000),100),10)+1),IF(MOD(MOD(INT($A16),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A16),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A16),1000),100)+1))))))&amp;" so'm"))</f>
+        <f>IF($A16="","",IF(INT($A16)=0,"nol so'm",TRIM(IF($D16&gt;0,$H16&amp;" milliard ","")&amp;IF($E16&gt;0,$I16&amp;" million ","")&amp;IF($F16&gt;0,$J16&amp;" ming ","")&amp;$K16)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D16" s="21">
+        <f>IF($A16="","",INT(INT($A16)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E16" s="21">
+        <f>IF($A16="","",INT(MOD(INT($A16),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F16" s="21">
+        <f>IF($A16="","",INT(MOD(INT($A16),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G16" s="21">
+        <f>IF($A16="","",MOD(INT($A16),1000))</f>
+        <v/>
+      </c>
+      <c r="H16" s="21">
+        <f>IF($A16="","",IF($D16=0,"",TRIM(IF(INT($D16/100)&gt;0,INDEX($N$4:$N$13,INT($D16/100)+1)&amp;" yuz ","")&amp;IF(MOD($D16,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D16,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D16,100),10)+1),IF(MOD($D16,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D16,100)-10+1),INDEX($N$4:$N$13,MOD($D16,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I16" s="21">
+        <f>IF($A16="","",IF($E16=0,"",TRIM(IF(INT($E16/100)&gt;0,INDEX($N$4:$N$13,INT($E16/100)+1)&amp;" yuz ","")&amp;IF(MOD($E16,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E16,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E16,100),10)+1),IF(MOD($E16,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E16,100)-10+1),INDEX($N$4:$N$13,MOD($E16,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J16" s="21">
+        <f>IF($A16="","",IF($F16=0,"",TRIM(IF(INT($F16/100)&gt;0,INDEX($N$4:$N$13,INT($F16/100)+1)&amp;" yuz ","")&amp;IF(MOD($F16,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F16,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F16,100),10)+1),IF(MOD($F16,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F16,100)-10+1),INDEX($N$4:$N$13,MOD($F16,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K16" s="21">
+        <f>IF($A16="","",IF($G16=0,"",TRIM(IF(INT($G16/100)&gt;0,INDEX($N$4:$N$13,INT($G16/100)+1)&amp;" yuz ","")&amp;IF(MOD($G16,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G16,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G16,100),10)+1),IF(MOD($G16,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G16,100)-10+1),INDEX($N$4:$N$13,MOD($G16,100)+1))))))</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n"/>
       <c r="B17" s="10">
-        <f>IF($A17="","",IF(INT($A17)=0,"nol so'm",TRIM(IF(INT(INT($A17)/1000000000)&gt;0,IF(INT(INT($A17)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A17)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A17)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A17)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A17)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A17)/1000000000),100),10)+1),IF(MOD(INT(INT($A17)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A17)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A17)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A17),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A17),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A17),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A17),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A17),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A17),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A17),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A17),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A17),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A17),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A17),1000000)/1000)&gt;0,IF(INT(MOD(INT($A17),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A17),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A17),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A17),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A17),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A17),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A17),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A17),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A17),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A17),1000)=0,"",TRIM(IF(INT(MOD(INT($A17),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A17),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A17),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A17),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A17),1000),100),10)+1),IF(MOD(MOD(INT($A17),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A17),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A17),1000),100)+1))))))&amp;" so'm"))</f>
+        <f>IF($A17="","",IF(INT($A17)=0,"nol so'm",TRIM(IF($D17&gt;0,$H17&amp;" milliard ","")&amp;IF($E17&gt;0,$I17&amp;" million ","")&amp;IF($F17&gt;0,$J17&amp;" ming ","")&amp;$K17)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D17" s="21">
+        <f>IF($A17="","",INT(INT($A17)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E17" s="21">
+        <f>IF($A17="","",INT(MOD(INT($A17),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F17" s="21">
+        <f>IF($A17="","",INT(MOD(INT($A17),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G17" s="21">
+        <f>IF($A17="","",MOD(INT($A17),1000))</f>
+        <v/>
+      </c>
+      <c r="H17" s="21">
+        <f>IF($A17="","",IF($D17=0,"",TRIM(IF(INT($D17/100)&gt;0,INDEX($N$4:$N$13,INT($D17/100)+1)&amp;" yuz ","")&amp;IF(MOD($D17,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D17,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D17,100),10)+1),IF(MOD($D17,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D17,100)-10+1),INDEX($N$4:$N$13,MOD($D17,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I17" s="21">
+        <f>IF($A17="","",IF($E17=0,"",TRIM(IF(INT($E17/100)&gt;0,INDEX($N$4:$N$13,INT($E17/100)+1)&amp;" yuz ","")&amp;IF(MOD($E17,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E17,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E17,100),10)+1),IF(MOD($E17,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E17,100)-10+1),INDEX($N$4:$N$13,MOD($E17,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J17" s="21">
+        <f>IF($A17="","",IF($F17=0,"",TRIM(IF(INT($F17/100)&gt;0,INDEX($N$4:$N$13,INT($F17/100)+1)&amp;" yuz ","")&amp;IF(MOD($F17,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F17,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F17,100),10)+1),IF(MOD($F17,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F17,100)-10+1),INDEX($N$4:$N$13,MOD($F17,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K17" s="21">
+        <f>IF($A17="","",IF($G17=0,"",TRIM(IF(INT($G17/100)&gt;0,INDEX($N$4:$N$13,INT($G17/100)+1)&amp;" yuz ","")&amp;IF(MOD($G17,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G17,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G17,100),10)+1),IF(MOD($G17,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G17,100)-10+1),INDEX($N$4:$N$13,MOD($G17,100)+1))))))</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n"/>
       <c r="B18" s="10">
-        <f>IF($A18="","",IF(INT($A18)=0,"nol so'm",TRIM(IF(INT(INT($A18)/1000000000)&gt;0,IF(INT(INT($A18)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A18)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A18)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A18)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A18)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A18)/1000000000),100),10)+1),IF(MOD(INT(INT($A18)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A18)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A18)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A18),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A18),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A18),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A18),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A18),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A18),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A18),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A18),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A18),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A18),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A18),1000000)/1000)&gt;0,IF(INT(MOD(INT($A18),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A18),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A18),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A18),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A18),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A18),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A18),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A18),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A18),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A18),1000)=0,"",TRIM(IF(INT(MOD(INT($A18),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A18),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A18),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A18),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A18),1000),100),10)+1),IF(MOD(MOD(INT($A18),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A18),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A18),1000),100)+1))))))&amp;" so'm"))</f>
+        <f>IF($A18="","",IF(INT($A18)=0,"nol so'm",TRIM(IF($D18&gt;0,$H18&amp;" milliard ","")&amp;IF($E18&gt;0,$I18&amp;" million ","")&amp;IF($F18&gt;0,$J18&amp;" ming ","")&amp;$K18)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D18" s="21">
+        <f>IF($A18="","",INT(INT($A18)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E18" s="21">
+        <f>IF($A18="","",INT(MOD(INT($A18),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F18" s="21">
+        <f>IF($A18="","",INT(MOD(INT($A18),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G18" s="21">
+        <f>IF($A18="","",MOD(INT($A18),1000))</f>
+        <v/>
+      </c>
+      <c r="H18" s="21">
+        <f>IF($A18="","",IF($D18=0,"",TRIM(IF(INT($D18/100)&gt;0,INDEX($N$4:$N$13,INT($D18/100)+1)&amp;" yuz ","")&amp;IF(MOD($D18,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D18,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D18,100),10)+1),IF(MOD($D18,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D18,100)-10+1),INDEX($N$4:$N$13,MOD($D18,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I18" s="21">
+        <f>IF($A18="","",IF($E18=0,"",TRIM(IF(INT($E18/100)&gt;0,INDEX($N$4:$N$13,INT($E18/100)+1)&amp;" yuz ","")&amp;IF(MOD($E18,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E18,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E18,100),10)+1),IF(MOD($E18,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E18,100)-10+1),INDEX($N$4:$N$13,MOD($E18,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J18" s="21">
+        <f>IF($A18="","",IF($F18=0,"",TRIM(IF(INT($F18/100)&gt;0,INDEX($N$4:$N$13,INT($F18/100)+1)&amp;" yuz ","")&amp;IF(MOD($F18,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F18,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F18,100),10)+1),IF(MOD($F18,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F18,100)-10+1),INDEX($N$4:$N$13,MOD($F18,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K18" s="21">
+        <f>IF($A18="","",IF($G18=0,"",TRIM(IF(INT($G18/100)&gt;0,INDEX($N$4:$N$13,INT($G18/100)+1)&amp;" yuz ","")&amp;IF(MOD($G18,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G18,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G18,100),10)+1),IF(MOD($G18,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G18,100)-10+1),INDEX($N$4:$N$13,MOD($G18,100)+1))))))</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n"/>
       <c r="B19" s="10">
-        <f>IF($A19="","",IF(INT($A19)=0,"nol so'm",TRIM(IF(INT(INT($A19)/1000000000)&gt;0,IF(INT(INT($A19)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A19)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A19)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A19)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A19)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A19)/1000000000),100),10)+1),IF(MOD(INT(INT($A19)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A19)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A19)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A19),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A19),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A19),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A19),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A19),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A19),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A19),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A19),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A19),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A19),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A19),1000000)/1000)&gt;0,IF(INT(MOD(INT($A19),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A19),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A19),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A19),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A19),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A19),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A19),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A19),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A19),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A19),1000)=0,"",TRIM(IF(INT(MOD(INT($A19),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A19),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A19),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A19),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A19),1000),100),10)+1),IF(MOD(MOD(INT($A19),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A19),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A19),1000),100)+1))))))&amp;" so'm"))</f>
+        <f>IF($A19="","",IF(INT($A19)=0,"nol so'm",TRIM(IF($D19&gt;0,$H19&amp;" milliard ","")&amp;IF($E19&gt;0,$I19&amp;" million ","")&amp;IF($F19&gt;0,$J19&amp;" ming ","")&amp;$K19)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D19" s="21">
+        <f>IF($A19="","",INT(INT($A19)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E19" s="21">
+        <f>IF($A19="","",INT(MOD(INT($A19),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F19" s="21">
+        <f>IF($A19="","",INT(MOD(INT($A19),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G19" s="21">
+        <f>IF($A19="","",MOD(INT($A19),1000))</f>
+        <v/>
+      </c>
+      <c r="H19" s="21">
+        <f>IF($A19="","",IF($D19=0,"",TRIM(IF(INT($D19/100)&gt;0,INDEX($N$4:$N$13,INT($D19/100)+1)&amp;" yuz ","")&amp;IF(MOD($D19,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D19,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D19,100),10)+1),IF(MOD($D19,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D19,100)-10+1),INDEX($N$4:$N$13,MOD($D19,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I19" s="21">
+        <f>IF($A19="","",IF($E19=0,"",TRIM(IF(INT($E19/100)&gt;0,INDEX($N$4:$N$13,INT($E19/100)+1)&amp;" yuz ","")&amp;IF(MOD($E19,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E19,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E19,100),10)+1),IF(MOD($E19,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E19,100)-10+1),INDEX($N$4:$N$13,MOD($E19,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J19" s="21">
+        <f>IF($A19="","",IF($F19=0,"",TRIM(IF(INT($F19/100)&gt;0,INDEX($N$4:$N$13,INT($F19/100)+1)&amp;" yuz ","")&amp;IF(MOD($F19,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F19,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F19,100),10)+1),IF(MOD($F19,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F19,100)-10+1),INDEX($N$4:$N$13,MOD($F19,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K19" s="21">
+        <f>IF($A19="","",IF($G19=0,"",TRIM(IF(INT($G19/100)&gt;0,INDEX($N$4:$N$13,INT($G19/100)+1)&amp;" yuz ","")&amp;IF(MOD($G19,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G19,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G19,100),10)+1),IF(MOD($G19,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G19,100)-10+1),INDEX($N$4:$N$13,MOD($G19,100)+1))))))</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n"/>
       <c r="B20" s="10">
-        <f>IF($A20="","",IF(INT($A20)=0,"nol so'm",TRIM(IF(INT(INT($A20)/1000000000)&gt;0,IF(INT(INT($A20)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A20)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A20)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A20)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A20)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A20)/1000000000),100),10)+1),IF(MOD(INT(INT($A20)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A20)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A20)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A20),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A20),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A20),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A20),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A20),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A20),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A20),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A20),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A20),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A20),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A20),1000000)/1000)&gt;0,IF(INT(MOD(INT($A20),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A20),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A20),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A20),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A20),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A20),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A20),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A20),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A20),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A20),1000)=0,"",TRIM(IF(INT(MOD(INT($A20),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A20),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A20),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A20),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A20),1000),100),10)+1),IF(MOD(MOD(INT($A20),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A20),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A20),1000),100)+1))))))&amp;" so'm"))</f>
+        <f>IF($A20="","",IF(INT($A20)=0,"nol so'm",TRIM(IF($D20&gt;0,$H20&amp;" milliard ","")&amp;IF($E20&gt;0,$I20&amp;" million ","")&amp;IF($F20&gt;0,$J20&amp;" ming ","")&amp;$K20)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D20" s="21">
+        <f>IF($A20="","",INT(INT($A20)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E20" s="21">
+        <f>IF($A20="","",INT(MOD(INT($A20),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F20" s="21">
+        <f>IF($A20="","",INT(MOD(INT($A20),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G20" s="21">
+        <f>IF($A20="","",MOD(INT($A20),1000))</f>
+        <v/>
+      </c>
+      <c r="H20" s="21">
+        <f>IF($A20="","",IF($D20=0,"",TRIM(IF(INT($D20/100)&gt;0,INDEX($N$4:$N$13,INT($D20/100)+1)&amp;" yuz ","")&amp;IF(MOD($D20,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D20,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D20,100),10)+1),IF(MOD($D20,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D20,100)-10+1),INDEX($N$4:$N$13,MOD($D20,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I20" s="21">
+        <f>IF($A20="","",IF($E20=0,"",TRIM(IF(INT($E20/100)&gt;0,INDEX($N$4:$N$13,INT($E20/100)+1)&amp;" yuz ","")&amp;IF(MOD($E20,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E20,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E20,100),10)+1),IF(MOD($E20,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E20,100)-10+1),INDEX($N$4:$N$13,MOD($E20,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J20" s="21">
+        <f>IF($A20="","",IF($F20=0,"",TRIM(IF(INT($F20/100)&gt;0,INDEX($N$4:$N$13,INT($F20/100)+1)&amp;" yuz ","")&amp;IF(MOD($F20,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F20,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F20,100),10)+1),IF(MOD($F20,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F20,100)-10+1),INDEX($N$4:$N$13,MOD($F20,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K20" s="21">
+        <f>IF($A20="","",IF($G20=0,"",TRIM(IF(INT($G20/100)&gt;0,INDEX($N$4:$N$13,INT($G20/100)+1)&amp;" yuz ","")&amp;IF(MOD($G20,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G20,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G20,100),10)+1),IF(MOD($G20,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G20,100)-10+1),INDEX($N$4:$N$13,MOD($G20,100)+1))))))</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n"/>
       <c r="B21" s="10">
-        <f>IF($A21="","",IF(INT($A21)=0,"nol so'm",TRIM(IF(INT(INT($A21)/1000000000)&gt;0,IF(INT(INT($A21)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A21)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A21)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A21)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A21)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A21)/1000000000),100),10)+1),IF(MOD(INT(INT($A21)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A21)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A21)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A21),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A21),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A21),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A21),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A21),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A21),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A21),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A21),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A21),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A21),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A21),1000000)/1000)&gt;0,IF(INT(MOD(INT($A21),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A21),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A21),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A21),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A21),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A21),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A21),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A21),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A21),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A21),1000)=0,"",TRIM(IF(INT(MOD(INT($A21),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A21),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A21),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A21),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A21),1000),100),10)+1),IF(MOD(MOD(INT($A21),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A21),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A21),1000),100)+1))))))&amp;" so'm"))</f>
+        <f>IF($A21="","",IF(INT($A21)=0,"nol so'm",TRIM(IF($D21&gt;0,$H21&amp;" milliard ","")&amp;IF($E21&gt;0,$I21&amp;" million ","")&amp;IF($F21&gt;0,$J21&amp;" ming ","")&amp;$K21)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D21" s="21">
+        <f>IF($A21="","",INT(INT($A21)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E21" s="21">
+        <f>IF($A21="","",INT(MOD(INT($A21),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F21" s="21">
+        <f>IF($A21="","",INT(MOD(INT($A21),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G21" s="21">
+        <f>IF($A21="","",MOD(INT($A21),1000))</f>
+        <v/>
+      </c>
+      <c r="H21" s="21">
+        <f>IF($A21="","",IF($D21=0,"",TRIM(IF(INT($D21/100)&gt;0,INDEX($N$4:$N$13,INT($D21/100)+1)&amp;" yuz ","")&amp;IF(MOD($D21,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D21,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D21,100),10)+1),IF(MOD($D21,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D21,100)-10+1),INDEX($N$4:$N$13,MOD($D21,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I21" s="21">
+        <f>IF($A21="","",IF($E21=0,"",TRIM(IF(INT($E21/100)&gt;0,INDEX($N$4:$N$13,INT($E21/100)+1)&amp;" yuz ","")&amp;IF(MOD($E21,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E21,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E21,100),10)+1),IF(MOD($E21,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E21,100)-10+1),INDEX($N$4:$N$13,MOD($E21,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J21" s="21">
+        <f>IF($A21="","",IF($F21=0,"",TRIM(IF(INT($F21/100)&gt;0,INDEX($N$4:$N$13,INT($F21/100)+1)&amp;" yuz ","")&amp;IF(MOD($F21,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F21,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F21,100),10)+1),IF(MOD($F21,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F21,100)-10+1),INDEX($N$4:$N$13,MOD($F21,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K21" s="21">
+        <f>IF($A21="","",IF($G21=0,"",TRIM(IF(INT($G21/100)&gt;0,INDEX($N$4:$N$13,INT($G21/100)+1)&amp;" yuz ","")&amp;IF(MOD($G21,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G21,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G21,100),10)+1),IF(MOD($G21,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G21,100)-10+1),INDEX($N$4:$N$13,MOD($G21,100)+1))))))</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n"/>
       <c r="B22" s="10">
-        <f>IF($A22="","",IF(INT($A22)=0,"nol so'm",TRIM(IF(INT(INT($A22)/1000000000)&gt;0,IF(INT(INT($A22)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A22)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A22)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A22)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A22)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A22)/1000000000),100),10)+1),IF(MOD(INT(INT($A22)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A22)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A22)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A22),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A22),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A22),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A22),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A22),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A22),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A22),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A22),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A22),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A22),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A22),1000000)/1000)&gt;0,IF(INT(MOD(INT($A22),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A22),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A22),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A22),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A22),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A22),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A22),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A22),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A22),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A22),1000)=0,"",TRIM(IF(INT(MOD(INT($A22),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A22),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A22),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A22),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A22),1000),100),10)+1),IF(MOD(MOD(INT($A22),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A22),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A22),1000),100)+1))))))&amp;" so'm"))</f>
+        <f>IF($A22="","",IF(INT($A22)=0,"nol so'm",TRIM(IF($D22&gt;0,$H22&amp;" milliard ","")&amp;IF($E22&gt;0,$I22&amp;" million ","")&amp;IF($F22&gt;0,$J22&amp;" ming ","")&amp;$K22)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D22" s="21">
+        <f>IF($A22="","",INT(INT($A22)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E22" s="21">
+        <f>IF($A22="","",INT(MOD(INT($A22),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F22" s="21">
+        <f>IF($A22="","",INT(MOD(INT($A22),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G22" s="21">
+        <f>IF($A22="","",MOD(INT($A22),1000))</f>
+        <v/>
+      </c>
+      <c r="H22" s="21">
+        <f>IF($A22="","",IF($D22=0,"",TRIM(IF(INT($D22/100)&gt;0,INDEX($N$4:$N$13,INT($D22/100)+1)&amp;" yuz ","")&amp;IF(MOD($D22,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D22,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D22,100),10)+1),IF(MOD($D22,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D22,100)-10+1),INDEX($N$4:$N$13,MOD($D22,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I22" s="21">
+        <f>IF($A22="","",IF($E22=0,"",TRIM(IF(INT($E22/100)&gt;0,INDEX($N$4:$N$13,INT($E22/100)+1)&amp;" yuz ","")&amp;IF(MOD($E22,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E22,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E22,100),10)+1),IF(MOD($E22,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E22,100)-10+1),INDEX($N$4:$N$13,MOD($E22,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J22" s="21">
+        <f>IF($A22="","",IF($F22=0,"",TRIM(IF(INT($F22/100)&gt;0,INDEX($N$4:$N$13,INT($F22/100)+1)&amp;" yuz ","")&amp;IF(MOD($F22,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F22,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F22,100),10)+1),IF(MOD($F22,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F22,100)-10+1),INDEX($N$4:$N$13,MOD($F22,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K22" s="21">
+        <f>IF($A22="","",IF($G22=0,"",TRIM(IF(INT($G22/100)&gt;0,INDEX($N$4:$N$13,INT($G22/100)+1)&amp;" yuz ","")&amp;IF(MOD($G22,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G22,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G22,100),10)+1),IF(MOD($G22,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G22,100)-10+1),INDEX($N$4:$N$13,MOD($G22,100)+1))))))</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
       <c r="B23" s="10">
-        <f>IF($A23="","",IF(INT($A23)=0,"nol so'm",TRIM(IF(INT(INT($A23)/1000000000)&gt;0,IF(INT(INT($A23)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A23)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A23)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A23)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A23)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A23)/1000000000),100),10)+1),IF(MOD(INT(INT($A23)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A23)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A23)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A23),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A23),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A23),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A23),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A23),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A23),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A23),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A23),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A23),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A23),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A23),1000000)/1000)&gt;0,IF(INT(MOD(INT($A23),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A23),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A23),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A23),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A23),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A23),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A23),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A23),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A23),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A23),1000)=0,"",TRIM(IF(INT(MOD(INT($A23),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A23),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A23),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A23),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A23),1000),100),10)+1),IF(MOD(MOD(INT($A23),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A23),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A23),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="20" t="n"/>
-      <c r="B24" s="10">
-        <f>IF($A24="","",IF(INT($A24)=0,"nol so'm",TRIM(IF(INT(INT($A24)/1000000000)&gt;0,IF(INT(INT($A24)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A24)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A24)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A24)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A24)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A24)/1000000000),100),10)+1),IF(MOD(INT(INT($A24)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A24)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A24)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A24),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A24),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A24),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A24),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A24),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A24),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A24),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A24),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A24),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A24),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A24),1000000)/1000)&gt;0,IF(INT(MOD(INT($A24),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A24),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A24),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A24),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A24),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A24),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A24),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A24),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A24),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A24),1000)=0,"",TRIM(IF(INT(MOD(INT($A24),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A24),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A24),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A24),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A24),1000),100),10)+1),IF(MOD(MOD(INT($A24),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A24),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A24),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="20" t="n"/>
-      <c r="B25" s="10">
-        <f>IF($A25="","",IF(INT($A25)=0,"nol so'm",TRIM(IF(INT(INT($A25)/1000000000)&gt;0,IF(INT(INT($A25)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A25)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A25)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A25)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A25)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A25)/1000000000),100),10)+1),IF(MOD(INT(INT($A25)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A25)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A25)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A25),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A25),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A25),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A25),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A25),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A25),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A25),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A25),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A25),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A25),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A25),1000000)/1000)&gt;0,IF(INT(MOD(INT($A25),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A25),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A25),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A25),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A25),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A25),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A25),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A25),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A25),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A25),1000)=0,"",TRIM(IF(INT(MOD(INT($A25),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A25),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A25),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A25),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A25),1000),100),10)+1),IF(MOD(MOD(INT($A25),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A25),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A25),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="20" t="n"/>
-      <c r="B26" s="10">
-        <f>IF($A26="","",IF(INT($A26)=0,"nol so'm",TRIM(IF(INT(INT($A26)/1000000000)&gt;0,IF(INT(INT($A26)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A26)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A26)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A26)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A26)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A26)/1000000000),100),10)+1),IF(MOD(INT(INT($A26)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A26)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A26)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A26),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A26),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A26),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A26),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A26),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A26),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A26),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A26),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A26),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A26),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A26),1000000)/1000)&gt;0,IF(INT(MOD(INT($A26),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A26),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A26),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A26),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A26),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A26),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A26),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A26),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A26),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A26),1000)=0,"",TRIM(IF(INT(MOD(INT($A26),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A26),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A26),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A26),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A26),1000),100),10)+1),IF(MOD(MOD(INT($A26),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A26),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A26),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="20" t="n"/>
-      <c r="B27" s="10">
-        <f>IF($A27="","",IF(INT($A27)=0,"nol so'm",TRIM(IF(INT(INT($A27)/1000000000)&gt;0,IF(INT(INT($A27)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A27)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A27)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A27)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A27)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A27)/1000000000),100),10)+1),IF(MOD(INT(INT($A27)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A27)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A27)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A27),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A27),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A27),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A27),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A27),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A27),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A27),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A27),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A27),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A27),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A27),1000000)/1000)&gt;0,IF(INT(MOD(INT($A27),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A27),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A27),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A27),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A27),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A27),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A27),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A27),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A27),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A27),1000)=0,"",TRIM(IF(INT(MOD(INT($A27),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A27),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A27),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A27),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A27),1000),100),10)+1),IF(MOD(MOD(INT($A27),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A27),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A27),1000),100)+1))))))&amp;" so'm"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="20" t="n"/>
-      <c r="B28" s="10">
-        <f>IF($A28="","",IF(INT($A28)=0,"nol so'm",TRIM(IF(INT(INT($A28)/1000000000)&gt;0,IF(INT(INT($A28)/1000000000)=0,"",TRIM(IF(INT(INT(INT($A28)/1000000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(INT($A28)/1000000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(INT($A28)/1000000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(INT($A28)/1000000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(INT($A28)/1000000000),100),10)+1),IF(MOD(INT(INT($A28)/1000000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(INT($A28)/1000000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(INT($A28)/1000000000),100)+1)))))&amp;" milliard ","")&amp;IF(INT(MOD(INT($A28),1000000000)/1000000)&gt;0,IF(INT(MOD(INT($A28),1000000000)/1000000)=0,"",TRIM(IF(INT(INT(MOD(INT($A28),1000000000)/1000000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A28),1000000000)/1000000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A28),1000000000)/1000000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A28),1000000000)/1000000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A28),1000000000)/1000000),100),10)+1),IF(MOD(INT(MOD(INT($A28),1000000000)/1000000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A28),1000000000)/1000000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A28),1000000000)/1000000),100)+1)))))&amp;" million ","")&amp;IF(INT(MOD(INT($A28),1000000)/1000)&gt;0,IF(INT(MOD(INT($A28),1000000)/1000)=0,"",TRIM(IF(INT(INT(MOD(INT($A28),1000000)/1000)/100)&gt;0,INDEX($I$4:$I$13,INT(INT(MOD(INT($A28),1000000)/1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(INT(MOD(INT($A28),1000000)/1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(INT(MOD(INT($A28),1000000)/1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(INT(MOD(INT($A28),1000000)/1000),100),10)+1),IF(MOD(INT(MOD(INT($A28),1000000)/1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(INT(MOD(INT($A28),1000000)/1000),100)-10+1),INDEX($I$4:$I$13,MOD(INT(MOD(INT($A28),1000000)/1000),100)+1)))))&amp;" ming ","")&amp;IF(MOD(INT($A28),1000)=0,"",TRIM(IF(INT(MOD(INT($A28),1000)/100)&gt;0,INDEX($I$4:$I$13,INT(MOD(INT($A28),1000)/100)+1)&amp;" yuz ","")&amp;IF(MOD(MOD(INT($A28),1000),100)&gt;=20,INDEX($J$4:$J$13,INT(MOD(MOD(INT($A28),1000),100)/10)+1)&amp;" "&amp;INDEX($I$4:$I$13,MOD(MOD(MOD(INT($A28),1000),100),10)+1),IF(MOD(MOD(INT($A28),1000),100)&gt;=10,"o'n "&amp;INDEX($I$4:$I$13,MOD(MOD(INT($A28),1000),100)-10+1),INDEX($I$4:$I$13,MOD(MOD(INT($A28),1000),100)+1))))))&amp;" so'm"))</f>
+        <f>IF($A23="","",IF(INT($A23)=0,"nol so'm",TRIM(IF($D23&gt;0,$H23&amp;" milliard ","")&amp;IF($E23&gt;0,$I23&amp;" million ","")&amp;IF($F23&gt;0,$J23&amp;" ming ","")&amp;$K23)&amp;" so'm"))</f>
+        <v/>
+      </c>
+      <c r="D23" s="21">
+        <f>IF($A23="","",INT(INT($A23)/1000000000))</f>
+        <v/>
+      </c>
+      <c r="E23" s="21">
+        <f>IF($A23="","",INT(MOD(INT($A23),1000000000)/1000000))</f>
+        <v/>
+      </c>
+      <c r="F23" s="21">
+        <f>IF($A23="","",INT(MOD(INT($A23),1000000)/1000))</f>
+        <v/>
+      </c>
+      <c r="G23" s="21">
+        <f>IF($A23="","",MOD(INT($A23),1000))</f>
+        <v/>
+      </c>
+      <c r="H23" s="21">
+        <f>IF($A23="","",IF($D23=0,"",TRIM(IF(INT($D23/100)&gt;0,INDEX($N$4:$N$13,INT($D23/100)+1)&amp;" yuz ","")&amp;IF(MOD($D23,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($D23,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($D23,100),10)+1),IF(MOD($D23,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($D23,100)-10+1),INDEX($N$4:$N$13,MOD($D23,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="I23" s="21">
+        <f>IF($A23="","",IF($E23=0,"",TRIM(IF(INT($E23/100)&gt;0,INDEX($N$4:$N$13,INT($E23/100)+1)&amp;" yuz ","")&amp;IF(MOD($E23,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($E23,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($E23,100),10)+1),IF(MOD($E23,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($E23,100)-10+1),INDEX($N$4:$N$13,MOD($E23,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="J23" s="21">
+        <f>IF($A23="","",IF($F23=0,"",TRIM(IF(INT($F23/100)&gt;0,INDEX($N$4:$N$13,INT($F23/100)+1)&amp;" yuz ","")&amp;IF(MOD($F23,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($F23,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($F23,100),10)+1),IF(MOD($F23,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($F23,100)-10+1),INDEX($N$4:$N$13,MOD($F23,100)+1))))))</f>
+        <v/>
+      </c>
+      <c r="K23" s="21">
+        <f>IF($A23="","",IF($G23=0,"",TRIM(IF(INT($G23/100)&gt;0,INDEX($N$4:$N$13,INT($G23/100)+1)&amp;" yuz ","")&amp;IF(MOD($G23,100)&gt;=20,INDEX($O$4:$O$13,INT(MOD($G23,100)/10)+1)&amp;" "&amp;INDEX($N$4:$N$13,MOD(MOD($G23,100),10)+1),IF(MOD($G23,100)&gt;=10,"o'n "&amp;INDEX($N$4:$N$13,MOD($G23,100)-10+1),INDEX($N$4:$N$13,MOD($G23,100)+1))))))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D3:K3"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>